<commit_message>
Added AI resumes + duplicates removed
</commit_message>
<xml_diff>
--- a/data/JDs.xlsx
+++ b/data/JDs.xlsx
@@ -1,42 +1,442 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\om\code\Resume-Evaluator\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2327CB0-C07D-40A1-B954-DAF29290DC8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="127">
-  <si>
-    <t>Category</t>
-  </si>
-  <si>
-    <t>Job Description</t>
-  </si>
-  <si>
-    <t>Data Science</t>
-  </si>
-  <si>
-    <t>Requirements
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
+</styleSheet>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B121"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Job Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Requirements
  Description and Requirements 
 Title: Data Partner - Computer Science
 Location: Asia - Remote
@@ -63,9 +463,18 @@
 At TELUS International, we enable customer experience innovation through spirited teamwork, agile thinking, and a caring culture that puts customers first. TELUS International is the global arm of TELUS Corporation, one of the largest telecommunications service providers in Canada. We deliver contact center and business process outsourcing (BPO) solutions to some of the world's largest corporations in the consumer electronics, finance, telecommunications and utilities sectors. With global call center delivery capabilities, our multi-shore, multi-language programs offer safe, secure infrastructure, value-based pricing, skills-based resources and exceptional customer service - all backed by TELUS, our multi-billion dollar telecommunications parent.
 Equal Opportunity Employer
 At TELUS International, we are proud to be an equal opportunity employer and are committed to creating a diverse and inclusive workplace. All aspects of employment, including the decision to hire and promote, are based on applicants’ qualifications, merits, competence and performance without regard to any characteristic related to diversity.</t>
-  </si>
-  <si>
-    <t>Way of working - Remote : Employees will have the freedom to work remotely all through the year. These employees, who form a large majority, will come together in their base location for a week, once every quarter.
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Way of working - Remote : Employees will have the freedom to work remotely all through the year. These employees, who form a large majority, will come together in their base location for a week, once every quarter.
 Job Profile: Data Scientist
 Location : Bangalore | Karnataka
 Years of Experience : 0 - 3
@@ -99,9 +508,18 @@
 https://bytes.swiggy.com/how-ai-at-swiggy-is-transforming-convenience-eae0a32055ae
 https://bytes.swiggy.com/decoding-food-intelligence-at-swiggy-5011e21dbc86
 We are an equal opportunity employer and all qualified applicants will receive consideration for employment without regard to race, colour, religion, sex, disability status, or any other characteristic protected by the law.</t>
-  </si>
-  <si>
-    <t>The ideal candidate's favorite words are learning, data, scale, and agility. You will leverage your strong collaboration skills and ability to extract valuable insights from highly complex data sets to ask the right questions and find the right answers.
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>The ideal candidate's favorite words are learning, data, scale, and agility. You will leverage your strong collaboration skills and ability to extract valuable insights from highly complex data sets to ask the right questions and find the right answers.
 Exp: 5 - 11 years
 Location: Across India
 Responsibilities
@@ -116,9 +534,18 @@
 Possess expertise in Natural Language Processing (NLP) &amp; GenAI to integrate text-based data sources into the Al architecture.
 Collaborate with data scientists and engineers to ensure seamless integration of Al components into existing systems.
 Responsible for continuous communication about the team progress to key stakeholder</t>
-  </si>
-  <si>
-    <t>Education: B.Tech/B.E. / MSc Statistics from premier institutes with minimum 80% marks in 10th and 12th grade or CGPA score of 7 and above in academics
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Education: B.Tech/B.E. / MSc Statistics from premier institutes with minimum 80% marks in 10th and 12th grade or CGPA score of 7 and above in academics
 Experience: 5 years
 Work timings: 2PM to 11 PM IST 
 Position Requirements: 
@@ -142,9 +569,18 @@
  ● Collaborate with cross-functional teams (marketing, product, engineering) to define project scope, objectives, and success metrics.
  ● Communicate complex technical findings to both technical and non-technical audiences.
  ● Stay abreast of the latest advancements in machine learning and data science, particularly in the healthcare domain.</t>
-  </si>
-  <si>
-    <t>About Searce
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>About Searce
 Searce is a cutting-edge tech consulting firm that empowers businesses to transform through Cloud, AI, and Analytics. We specialize in modernizing infrastructure, applications, and processes, enabling clients to achieve futuristic business outcomes. As a leading partner for Google Cloud and AWS, we are the trusted choice for tech startups and digital enterprises driving industry disruption.
 Job Responsibilities
 Understand business goals and develop models with measurable success metrics.
@@ -169,9 +605,18 @@
 Familiarity with data management, cloud computing, and big data platforms.
 Excellent communication skills for explaining complex solutions.
 Preference will be given to immediate joiners</t>
-  </si>
-  <si>
-    <t>What you’ll be doing (ie. job duties):
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>What you’ll be doing (ie. job duties):
 Mine and analyze products‘ user data. Work with the product team on using data to guide product strategy
 Write subgraph queries or APIs to curate on-chain and off-chain behavioral data
 Analyze different web3 protocols' on-chain data and write analysis report
@@ -188,9 +633,18 @@
 Excellent written and verbal communication skills
 A drive to learn and master new technologies and techniques
 Fluent in English and Mandarin</t>
-  </si>
-  <si>
-    <t>We are seeking a Staff Data Scientist to transform large datasets into actionable insights and new products for our fast-growth early stage company in the rideshare analytics space. You will lead the design and implementation of machine learning models and statistical analyses to support key business goals. In this role, you’ll drive data-driven decision-making, shape the company’s data science and machine learning capabilities, and effectively communicate complex technical concepts to diverse audiences with strong written and verbal communication skills.
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>We are seeking a Staff Data Scientist to transform large datasets into actionable insights and new products for our fast-growth early stage company in the rideshare analytics space. You will lead the design and implementation of machine learning models and statistical analyses to support key business goals. In this role, you’ll drive data-driven decision-making, shape the company’s data science and machine learning capabilities, and effectively communicate complex technical concepts to diverse audiences with strong written and verbal communication skills.
 We are willing to work on a contract to permanent hire basis.
 Day to Day Responsibilities:
 Evaluate machine learning opportunities and provide recommendations to address business needs and guide data science strategy.
@@ -215,9 +669,18 @@
 Strong project management skills to balance short-term tasks with long-term goals.
 Excellent written and verbal communication skills for explaining complex concepts to non-technical stakeholders.
 BS in Data Science, Statistics, Mathematics, Economics, Computer Science, Information Management, or equivalent experience.</t>
-  </si>
-  <si>
-    <t>Character.AI is building the future of open-ended interactions between people and intelligent agents. This requires rethinking design, user interfaces, and interactions from first principles.
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Character.AI is building the future of open-ended interactions between people and intelligent agents. This requires rethinking design, user interfaces, and interactions from first principles.
 We are seeking a talented and creative Data Scientist to join our team and play a pivotal role in shaping the user experience of our AI entertainment products. As a Product Designer, you will collaborate closely with cross-functional teams to design innovative, user-centered solutions that delight and inspire our customers. The ideal candidate will have a deep understanding of user-centric design, a strong portfolio showcasing their craft, and a passion for pushing the boundaries of what's possible with AI.
 What you’ll do:
 We are seeking a highly skilled and experienced Data Scientist with a strong background in consumer products to join our dynamic team. Experience working with open-ended, user-generated content is a major plus.
@@ -234,9 +697,18 @@
 In just two years, we achieved unicorn status and were honored as Google Play's AI App of the Year—a testament to our innovative technology and visionary approach.
 Join us and be a part of establishing this new entertainment paradigm while shaping the future of Consumer AI!
 At Character, we value diversity and welcome applicants from all backgrounds. As an equal opportunity employer, we firmly uphold a non-discrimination policy based on race, religion, national origin, gender, sexual orientation, age, veteran status, or disability. Your unique perspectives are vital to our success.</t>
-  </si>
-  <si>
-    <t>As a Senior Research Data Scientist, you will have end-to-end ownership of custom models, heuristics, algorithms, and other data products that feed directly into TRM’s UX. In collaboration with a highly skilled team of engineers, data scientists, and research scientists, your goal will be to uncover valuable and defensible information that can be used to detect, prevent, and mitigate cryptocurrency fraud and financial crime.
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>As a Senior Research Data Scientist, you will have end-to-end ownership of custom models, heuristics, algorithms, and other data products that feed directly into TRM’s UX. In collaboration with a highly skilled team of engineers, data scientists, and research scientists, your goal will be to uncover valuable and defensible information that can be used to detect, prevent, and mitigate cryptocurrency fraud and financial crime.
 The models and algorithms you create will be specifically designed to identify new threat vectors that are unique to cryptocurrencies and blockchains. These tools will be consumed by prestigious entities such as former FBI, Secret Service, and other law enforcement agencies, enabling them to stay ahead of evolving criminal activities in the cryptocurrency space.
 In particular, the Traceability Team is responsible for investigating and tracing illicit actors that utilize technologies intentionally designed to obscure their blockchain transactions. The problems we face are exciting, challenging, and open-ended, requiring strong research-minded focus and curiosity. If you like solving hard problems with smart people, this is the place for you!
 The impact you will have here:
@@ -266,9 +738,18 @@
 The following represents the expected range of compensation for this role:
 The estimated base salary range for this role is $170,000 - $190,000. Please note that the base range is applicable to the US and will be different depending on the country.
 Additionally, this role may be eligible to participate in TRM’s equity plan.</t>
-  </si>
-  <si>
-    <t>About Invoca
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>About Invoca
 Commitment to our customers, collaboration, and continuous improvement in a positive environment are more than words written on a wall at Invoca, it’s our way of life. We take pride in an inclusive and egoless culture that helps us drive innovation and build value for both our customers and our people. And of course, there’s the competitive pay, great perks, and getting to work on an industry-leading product. If this sounds unlike most tech jobs you’ve had, you’re right. Come join us. We’re building something special.
 About the Engineering Team
 You’ll join a team where everyone, including you, is striving to constantly improve their knowledge of software development tools, practices, and processes. We are an incredibly supportive team. We swarm when problems arise and give excellent feedback to help each other grow. Working on our close-knit, multi-functional teams is a chance to share and grow your knowledge of different domains from databases to front ends to telephony and everything in between.
@@ -323,9 +804,18 @@
 DEI Statement
 We are committed to equal employment opportunity regardless of race, color, ancestry, religion, sex, national origin, sexual orientation, age, citizenship, marital status, disability, gender, gender identity or expression, or veteran status. We are proud to be an equal opportunity workplace.
 #LI-Remote</t>
-  </si>
-  <si>
-    <t>About the Role
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>About the Role
 Location: Remote, United States
 Role Type: Full-Time
 Reports To: CPO
@@ -359,9 +849,18 @@
 Excellent communication and collaboration skills
 Ability to work in a fast-paced, startup environment
 Proactive, independent, responsible attitude with the ability to learn quickly</t>
-  </si>
-  <si>
-    <t>Job Description:
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Job Description:
 Intern - Data scientist/ Computer vision Research and development
 We are looking for Data Scientist Intern(s) who are currently pursuing undergraduate (BS), (MS)
 or PhD degree to join our research and analysis team. This team primarily focuses on conducting research and analysis to bring answers to the complex business problems using mathematical, statistical and predictive data modelling techniques which leads to the business decision that ensure senior safety and health.
@@ -378,9 +877,18 @@
 Experience in applying machine learning techniques and concepts to Computer vision problems.
 Collaborate with other teams and departments
 Willingness to learn new things very fast independently</t>
-  </si>
-  <si>
-    <t>About thirdweb
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>About thirdweb
 thirdweb is a full stack development platform for web3.
 We provide frontend, backend and on-chain tools for developers to build apps &amp; games that works on any EVM chain. Our mission is to empower developers to easily create decentralized internet products, and serve them to billions of users.
 Over 100,000 developers use thirdweb every month and over 1M unique wallets have interacted with our contracts on mainnet. Companies like Shopify, AWS, Coinbase, Circle, Rarible, Animoca Brands, and many more use our product to build and power their applications.
@@ -414,9 +922,18 @@
 🧘‍♂️ Workplace Wellbeing program
 👶 Parental Leave support
 ✈️ The ability to work remotely or in one of our stunning office spaces in Fort Mason, San Francisco and Williamsburg, Brooklyn.</t>
-  </si>
-  <si>
-    <t>Data Scientist
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Data Scientist
 Location: Fort Lauderdale / Remote
 Department: Data Science
 Reports To: Chief Technology Officer (CTO)
@@ -458,9 +975,18 @@
 How to Apply:
 If you are a driven and experienced data scientist looking to lead and make a significant impact, we would love to hear from you. Please submit your resume and a cover letter detailing your relevant experience.
 Please complete this assestment in order to interview https://app.testgorilla.com/s/segkopxz . Once completed email maria@getrevscale.com with a copy of your current resume.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Why TrueML?
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Why TrueML?
 TrueML is a mission-driven financial software company that aims to create better customer experiences for distressed borrowers. Consumers today want personal, digital-first experiences that align with their lifestyles, especially when it comes to managing finances. TrueML’s approach uses machine learning to engage each customer digitally and adjust strategies in real time in response to their interactions.
 The TrueML team includes inspired data scientists, financial services industry experts and customer experience fanatics building technology to serve people in a way that recognizes their unique needs and preferences as human beings and endeavoring toward ensuring nobody gets locked out of the financial system.
 The Role:
@@ -485,9 +1011,18 @@
 Our Dedication to Diversity &amp; Inclusion
 TrueML and TrueAccord are equal opportunity employers. We promote, value, and thrive with a diverse &amp; inclusive team. Different perspectives contribute to better solutions and this makes us stronger every day. We do not discriminate on the basis of race, religion, color, national origin, gender, sexual orientation, age, marital status, veteran status, or disability status.
 </t>
-  </si>
-  <si>
-    <t>We are based in Pune looking to hire interns for Data science program .
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>We are based in Pune looking to hire interns for Data science program .
 Skills: Python , Data Science , Machine Learning
 Interns can join us for College project .
 We are offering Hybrid internship also.
@@ -500,16 +1035,34 @@
 Education:
 Bachelor's (Preferred)
 Work Location: In person</t>
-  </si>
-  <si>
-    <t>Strong proficiency in programming languages such as Python and R.
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Strong proficiency in programming languages such as Python and R.
 Expertise in sentiment analysis, NER, and other natural language processing techniques is a must.
 Experience in MLOps, Machine Learning, Statistical Modeling, and Data Visualization.
 Excellent leadership, communication, and interpersonal skills.
 Number of Openings : 3</t>
-  </si>
-  <si>
-    <t>Optum AI is UnitedHealth Group’s enterprise AI team. We are AI/ML scientists and engineers with deep expertise in AI/ML engineering for health care. We develop AI/ML solutions for the highest impact opportunities across UnitedHealth Group businesses including UnitedHealthcare, Optum Financial, Optum Health, Optum Insight, and Optum Rx. In addition to transforming the health care journey through responsible AI/ML innovation, our charter also includes developing and supporting an enterprise AI/ML development platform.
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Optum AI is UnitedHealth Group’s enterprise AI team. We are AI/ML scientists and engineers with deep expertise in AI/ML engineering for health care. We develop AI/ML solutions for the highest impact opportunities across UnitedHealth Group businesses including UnitedHealthcare, Optum Financial, Optum Health, Optum Insight, and Optum Rx. In addition to transforming the health care journey through responsible AI/ML innovation, our charter also includes developing and supporting an enterprise AI/ML development platform.
 Optum AI team members:
 Have impact at scale: We have the data and resources to make an impact at scale. When our solutions are deployed, they have the potential to make health care system work better for everyone.
 Do ground-breaking work: Many of our current projects involve cutting edge ML, NLP and LLM techniques. Generative AI methods for working with structured and unstructured health care data are continuously being developed and improved. We are working in one of the most important frontiers of AI/ML research and development.
@@ -539,9 +1092,18 @@
 Proven exceptional verbal and written communication skills to relate with and supervise teams, as well as to communicate technical content and analytical insights/complex findings in a clear and concise manner to multiple audiences, including senior management
 At UnitedHealth Group, our mission is to help people live healthier lives and make the health system work better for everyone. We believe everyone–of every race, gender, sexuality, age, location and income–deserves the opportunity to live their healthiest life. Today, however, there are still far too many barriers to good health which are disproportionately experienced by people of color, historically marginalized groups and those with lower incomes. We are committed to mitigating our impact on the environment and enabling and delivering equitable care that addresses health disparities and improves health outcomes - an enterprise priority reflected in our mission. #nic
 #LETSGROW</t>
-  </si>
-  <si>
-    <t>Entity:
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Entity:
 Finance
 Job Family Group:
 Subsurface Group
@@ -589,9 +1151,18 @@
 Legal Disclaimer:
 We are an equal opportunity employer and value diversity at our company. We do not discriminate on the basis of race, religion, color, national origin, sex, gender, gender expression, sexual orientation, age, marital status, socioeconomic status, neurodiversity/neurocognitive functioning, veteran status or disability status. Individuals with an accessibility need may request an adjustment/accommodation related to bp’s recruiting process (e.g., accessing the job application, completing required assessments, participating in telephone screenings or interviews, etc.). If you would like to request an adjustment/accommodation related to the recruitment process, please contact us.
 If you are selected for a position and depending upon your role, your employment may be contingent upon adherence to local policy. This may include pre-placement drug screening, medical review of physical fitness for the role, and background checks.</t>
-  </si>
-  <si>
-    <t>Job Title
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Job Title
 Data Scientist 4
 Common accountabilities:
 Has working experience and advanced and specialized technical/functional knowledge in own discipline. Understands how own area contributes to the business. Acts as a reference for colleagues with less experience and supports junior team members.
@@ -608,12 +1179,18 @@
 Diversity &amp; Inclusion
 Amadeus aspires to be a leader in Diversity, Equity and Inclusion in the tech industry, enabling every employee to reach their full potential by fostering a culture of belonging and fair treatment, attracting the best talent from all backgrounds, and as a role model for an inclusive employee experience.
 Amadeus is an equal opportunity employer. All qualified applicants will receive consideration for employment without regard to gender, race, ethnicity, sexual orientation, age, beliefs, disability or any other characteristics protected by law.</t>
-  </si>
-  <si>
-    <t>Web Designing</t>
-  </si>
-  <si>
-    <t>Work closely with the onshore teams and clients while running and being responsible for multiple projects at the offshore development centre.
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Web Designing</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Work closely with the onshore teams and clients while running and being responsible for multiple projects at the offshore development centre.
 Conduct extensive automated unit testing of programs in Web and mobile software applications to ensure they will produce the desired outcome.
 Write and maintain standards for HTML, CSS or Javascript.
 Devise complex architectural front end functional elements.
@@ -637,9 +1214,18 @@
 Working experience with consuming REST APIs is an advantage.
 Expertise in effective design, responsive, secure and power-sensitive apps.
 Experience of web-based UI development for cross-browser support, progressive web apps.</t>
-  </si>
-  <si>
-    <t>Skill required: Marketing Operations - Creative Design
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Web Designing</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Skill required: Marketing Operations - Creative Design
 Designation: Motion Design Associate
 Qualifications:Any Graduation
 Years of Experience:1 to 3 years
@@ -682,9 +1268,18 @@
  Interprets sponsor s graphic requirements to maximize creativity and productivity; offer graphic solutions that support the project requirements or constraints.
  Creates a Visual Approach document as requested by a supervisor, including graphic proposals, animations and prototypes.
  Oversees and assists in issue resolution by utilizing all support resources available.</t>
-  </si>
-  <si>
-    <t>Skills:
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Web Designing</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Skills:
 Adobe Photoshop, Adobe Illustrator, UI/UX Design, Responsive Web Design, HTML/CSS, JavaScript, Sketch, Figma,
 Responsibilities
 Design and develop visually appealing websites that adhere to the latest design standards.
@@ -710,13 +1305,31 @@
 The interview process is currently being conducted in person, and we are focusing on local candidates from Surat.
 Desired Skills and Experience
 Adobe Photoshop, Adobe Illustrator, UI/UX Design, Responsive Web Design, HTML/CSS, JavaScript, Sketch, Figma</t>
-  </si>
-  <si>
-    <t>SummaryIn this role, you pride yourself on staying at the cutting edge of UI design and development. You are equally comfortable creating an interactive prototype, and developing maintainable CSS SASS LESS, HTML, and JavaScript. You believe that semantic markup, web accessibility and performance optimization are must haves on every page you deliver, and you devour articles describing ways to improve the quality of the user experience 6 to 8 years of experience in developing front end code for an enterprise content management system (eg Adobe Experience Manager, Sitecore.ResponsibilitiesProduce great front end code. You enjoy producing clean, easy to read, semantic HTML markup and CSS, adhering to W3C specs and best practices. Youre skilled at architecting modular, maintainable, and extensible CSS code. (Deep experiences with SASS a major plus.) You re also deeply familiar with jQuery and the best plugins.Leverage modular CSS methodologies like BEM, OOCSSDevelop new user-facing features based on provided designs and style systemBuild reusable code and libraries for future useOptimize front-end pages for maximum speed and scalability, with a focus on Core Web VitalsEnsure pages adhere to accessibility standards specifically WCAG 2.2 AA conformanceAssure that all user input is validated before submitting to back-endCollaborate with other team members and stakeholdersEnsure the application scales well across browsers (Cross Browser Testing)Build UI components using Storybook.Experience in using Figma a plusKey capabilitiesProficient understanding of web markup, including HTML5 and CSS3Proficient understanding of core web vitals and techniques for optimizing page load timesStrong knowledge of Twitter Bootstrap framework and Responsive Design using media queriesStrong background of frontend development tools such as npm and webpack.Basic understanding of server-side CSS pre-processing platforms, such as LESS and SASSExperience writing cross-browser and cross-platform markup, styles, and JavaScriptAbility to write custom JavaScript, as well as work with popular JavaScript tools such as jQueryCollaborate with cross functional teams to integrate UI components into a content management systemBasic understanding of AEMs Sightly HTLProficient in using Font, icons and implement using CSS3Conduct thorough testing of UI components to ensure compatibility and adherence o quality standardsProficient understanding of cross browser compatibility issues and ways to work around themFair understanding of JavaScript programming and DOM manipulationGood understanding of SEO principles and ensuring that the application will adhere to themProficient understanding of code versioning tools, such as Git
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Web Designing</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>SummaryIn this role, you pride yourself on staying at the cutting edge of UI design and development. You are equally comfortable creating an interactive prototype, and developing maintainable CSS SASS LESS, HTML, and JavaScript. You believe that semantic markup, web accessibility and performance optimization are must haves on every page you deliver, and you devour articles describing ways to improve the quality of the user experience 6 to 8 years of experience in developing front end code for an enterprise content management system (eg Adobe Experience Manager, Sitecore.ResponsibilitiesProduce great front end code. You enjoy producing clean, easy to read, semantic HTML markup and CSS, adhering to W3C specs and best practices. Youre skilled at architecting modular, maintainable, and extensible CSS code. (Deep experiences with SASS a major plus.) You re also deeply familiar with jQuery and the best plugins.Leverage modular CSS methodologies like BEM, OOCSSDevelop new user-facing features based on provided designs and style systemBuild reusable code and libraries for future useOptimize front-end pages for maximum speed and scalability, with a focus on Core Web VitalsEnsure pages adhere to accessibility standards specifically WCAG 2.2 AA conformanceAssure that all user input is validated before submitting to back-endCollaborate with other team members and stakeholdersEnsure the application scales well across browsers (Cross Browser Testing)Build UI components using Storybook.Experience in using Figma a plusKey capabilitiesProficient understanding of web markup, including HTML5 and CSS3Proficient understanding of core web vitals and techniques for optimizing page load timesStrong knowledge of Twitter Bootstrap framework and Responsive Design using media queriesStrong background of frontend development tools such as npm and webpack.Basic understanding of server-side CSS pre-processing platforms, such as LESS and SASSExperience writing cross-browser and cross-platform markup, styles, and JavaScriptAbility to write custom JavaScript, as well as work with popular JavaScript tools such as jQueryCollaborate with cross functional teams to integrate UI components into a content management systemBasic understanding of AEMs Sightly HTLProficient in using Font, icons and implement using CSS3Conduct thorough testing of UI components to ensure compatibility and adherence o quality standardsProficient understanding of cross browser compatibility issues and ways to work around themFair understanding of JavaScript programming and DOM manipulationGood understanding of SEO principles and ensuring that the application will adhere to themProficient understanding of code versioning tools, such as Git
 SVNProvide clear and comprehensive documentation for developed UI components.Effectively communicate with team members, stakeholders, and project managers.Experience in Agile development is a plusEducationBachelors degree in Computer Science, Engineering, or a related field.Adobe Experience Cloud related certifications preferred.</t>
-  </si>
-  <si>
-    <t>About the job
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Web Designing</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>About the job
 Greetings from TCS!!
 TCS is hiring for Webmethods Designer
 Job Title: Webmethods Designer
@@ -735,9 +1348,18 @@
 Knowledge in UML diagrams
 Should have basic knowledge on data base query and store procedure.
 Should have knowledge on various integration patterns</t>
-  </si>
-  <si>
-    <t>At Locker, we have created a consumer shopping platform that revolutionizes the way consumers shop, and is democratizing curation and affiliate earning for the everyday consumer. Locker was named among the top 5 commerce startups and among the top 50 startups in 2024 by The Information. We are a seed stage startup, and have raised $3.5M in funding, with our seed round led by Wonder Ventures.
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Web Designing</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>At Locker, we have created a consumer shopping platform that revolutionizes the way consumers shop, and is democratizing curation and affiliate earning for the everyday consumer. Locker was named among the top 5 commerce startups and among the top 50 startups in 2024 by The Information. We are a seed stage startup, and have raised $3.5M in funding, with our seed round led by Wonder Ventures.
 Locker is seeking a senior frontend engineer to join our team. In this role you will be responsible for delivering world-class UI to our user base, using your wide range of skills and expertise working in a product-driven organization.
 We are a remote team, mostly located in the Los Angeles area with occasional meetings on-site.
 Why join Locker’s Engineering team?
@@ -781,9 +1403,18 @@
 -Substantial equity stake in the startup, aligning your success with ours, competitive base salary, and health benefits.
 -The opportunity to shape the future of commerce with a diverse group of successful, talented and motivated colleagues.
 Apply now to join our team!</t>
-  </si>
-  <si>
-    <t>Please note:
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Web Designing</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Please note:
 We do not accept applications without a personalized note explaining your interest in and suitability for this particular role with us.
 Compensation varies based on the type of engagement. Independent contractors may have higher rates than employees due to differences in tax and benefit structures.
 Valory
@@ -827,9 +1458,18 @@
 You will work on a unique software stack and product with a team of world-class software engineers, researchers, and product experts across multiple fields.
 You will collaborate with teams across crypto and our community of agent developers.
 You will redefine how developers build off-chain services in DeFi and long into web3’s future.</t>
-  </si>
-  <si>
-    <t>Do you want to help make the world safe from cyber attack?
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Web Designing</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Do you want to help make the world safe from cyber attack?
 At Corelight, we believe that the best approach to cybersecurity risk starts with the network. Attackers can evade endpoint detection, firewalls and many other technologies - but they can’t avoid leaving digital footprints on the networks they traverse. Built on open-source innovations from Zeek, Suricata and YARA and refined through years of real-world use, Corelight transforms network footprints from physical, virtual and cloud networks into actionable insights. Our customers use these insights to speed incident response and proactively hunt for threats.
 As a Lead FullStack Engineer, you will play a crucial role in leading the development and architecture of the frontend systems that power our products and services. You will be responsible for overseeing a team of FullStack/UI engineers, guiding their work, and collaborating with cross-functional teams to deliver high-quality, scalable, and reliable software solutions. Your deep understanding of React, GraphQL and associated technologies, combined with your leadership skills, will be vital in shaping the future of Corelight's Open NDR SaaS Platform.
 Responsibilities
@@ -858,9 +1498,18 @@
 Experience working in a distributed team.
 Fueled by investments from top-tier venture capital organizations such as Crowdstrike, Accel and Insight, Corelight is the fastest growing network detection and response platform in the industry. Our customers trust us to protect mission-critical assets in leading enterprises, government, and research institutions worldwide. We are leading the way with AI-assisted workflows, machine learning models, cloud security and SaaS-based solutions to arm defenders with the tools and knowledge they need to disrupt cyber attacks. Our team of passionate innovators are dedicated to solving some of the toughest challenges in cybersecurity, while fostering a collaborative, inclusive, and growth-oriented culture. Corelight is committed to a geographically distributed yet connected employee base with employees working from home and office locations around the world. At Corelight, we are proud of our diversity of background and thought, and we’re united by our strong shared culture and values.
 We are looking forward to meeting you. Check us out at www.corelight.com</t>
-  </si>
-  <si>
-    <t>At Doist, our mission is to empower people with simple yet powerful tools.
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Web Designing</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>At Doist, our mission is to empower people with simple yet powerful tools.
 We're a multidisciplinary, fully-remote, team that’s passionate about creating products, like Todoist and Twist, that improve people’s lives. We thrive on innovating new solutions to old productivity challenges and we seek to rethink how productivity tools are made.
 Our Core Values
 They are few, but they are mighty. From creating processes to decision-making and recruiting, we build our four core values into nearly every single thing we do.
@@ -918,9 +1567,18 @@
 Invest in your health and wellness. Take care of yourself with a monthly budget for things like a gym membership, healthy snacks, massages, health insurance, etc.
 We occasionally receive reports about hiring scams related to our roles. Please be aware that our team only communicates from emails with an "@doist.com" domain and that we will not ask you to apply in any way other than via our application at doist.com/careers. If you are in doubt, please reach out at careers@doist.com to confirm.
 All information collected through this application is stored in Workable, Doist’s Applicant Tracking System, where it will be used for recruitment purposes only. For more information on how we handle candidate data at Doist, we invite you to review our recruitment privacy notice. For questions, please contact us at careers@doist.com.</t>
-  </si>
-  <si>
-    <t>About the Role:
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Web Designing</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>About the Role:
 We are seeking a highly skilled Senior Frontend Engineer to join our growing engineering team. The ideal candidate will have a passion for creating user-friendly web applications with great attention to detail and a strong background in modern frontend technologies.
 Key Responsibilities:
 Develop from scratch web applications for healthcare providers and patients.
@@ -931,9 +1589,18 @@
 Proficiency in HTML, CSS, TypeScript, and React.
 Experience with state management libraries.
 Experience with automated testing frameworks(e.g., Jest, Mocha).</t>
-  </si>
-  <si>
-    <t>Digify is a cloud-based document security and data room software that allows customers to control, protect and track important documents after sharing them. Companies use Digify to protect confidential information for fundraising and due diligence, secure intellectual property, and protect sensitive communications.
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Web Designing</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Digify is a cloud-based document security and data room software that allows customers to control, protect and track important documents after sharing them. Companies use Digify to protect confidential information for fundraising and due diligence, secure intellectual property, and protect sensitive communications.
 Digify is used in 138 countries today. We have more than 600,000 users worldwide.
 We are looking for a skilled Frontend Engineer with 3-5 years of experience to join our team. In this role, you will be responsible for developing and maintaining high-quality, scalable Angular applications while ensuring optimal performance and seamless integration with backend services.
 You should have a strong grasp of Angular, TypeScript, state management, UI libraries like Ant Design, and security best practices. Writing clean, maintainable, and testable code is a key part of this role, along with implementing unit tests using Jasmine, Karma, or Jest.
@@ -962,9 +1629,18 @@
 Experience mobile application development.
 Experience with Angular SSR &amp; performance optimization.
 Familiarity with Storybook &amp; component documentation.</t>
-  </si>
-  <si>
-    <t>About us.
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Web Designing</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>About us.
 Trumid is a dynamic fintech revolutionizing the landscape of fixed income trading. With intelligent, easy-to-use, electronic solutions, we are rapidly growing and seeking exceptional talent to help redefine the boundaries of technology and finance.
 Founded in 2014 by a team of fixed income market experts, Trumid has quickly become one of the top three corporate bond e-trading platforms in the U.S. Today, over 1,300 traders from an extensive and expanding client network of 920+ buy-and sell-side institutions transact on Trumid monthly.
 With a rich history of innovation and a unique ability to innovate at scale, we collaborate closely with our clients, iterating quickly toward optimal solutions. With market share and client engagement at all-time highs and our pace of product development faster than ever, this is an exciting and transformative time at Trumid.
@@ -992,16 +1668,34 @@
 Team-oriented and collaborative company culture
 Remote first
 Trumid is an equal opportunity employer.</t>
-  </si>
-  <si>
-    <t>We are a team of 5 incredibly driven and talented core members. We are looking for a frontend engineer who can keep up with us, and has the right energy and excitement to build a Unicorn with us. You must have 0-1/startup experience owning all of frontend development, deep expo + react native experience, and an insatiable drive to succeed and build. Our product is very design-heavy so if you have a keen eye and infatuation with pixel-perfect, clean UI development, you're in the right place. We are looking for a contractor to work on a retainer (full time hours for a couple months, as decided through further conversation together), with the potential to extend a full time founding frontend engineer offer by the end.
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Web Designing</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>We are a team of 5 incredibly driven and talented core members. We are looking for a frontend engineer who can keep up with us, and has the right energy and excitement to build a Unicorn with us. You must have 0-1/startup experience owning all of frontend development, deep expo + react native experience, and an insatiable drive to succeed and build. Our product is very design-heavy so if you have a keen eye and infatuation with pixel-perfect, clean UI development, you're in the right place. We are looking for a contractor to work on a retainer (full time hours for a couple months, as decided through further conversation together), with the potential to extend a full time founding frontend engineer offer by the end.
 What is ARI: We are building the next-gen clothing shopping experience. We built an AI-driven virtual avatar named ARI who shops for fashion items across the internet, personalized to users' style. ARI leverages our proprietary recommendation system that detects nuanced personal style through numerous variables as well as conducting sentiment analysis over chat-bot conversations. ARI returns personalized clothing product recommendations sourced across the entire internet through vector search for users.
 Partnered with industry giants William Morris Endeavor and IMG Models and backed by early investors such as Bloomberg Beta, 1517 VC, Z Fellows, co-founder of Venmo, CEO of Miss Universe, ex-CPO of Hinge, CS faculty @Stanford, AI/ML lead @ Apple, CTO of Linktree, ex-CMO of Bella Hadid’s Kin, @andrewyeung among others, we are positioned to win. We currently have an MVP built and are onboarding + collecting feedback from a small subset of our growing waitlist.
 Founder: Lior Cole dropped out of Cornell CS to build full-time, she is also a worldwide IMG Model. See her TedxCornell talk with a very early ARI chat demo here: https://www.youtube.com/watch?v=gCRcIbdaCDk
 Stack: expo + react native</t>
-  </si>
-  <si>
-    <t>As a Senior Frontend Developer at USDT0, you will play a key role in building and refining our user-facing products. You’ll work closely with designers, product managers, and backend engineers to create intuitive, high-performing, and scalable web applications that showcase the potential of stablecoins to a global audience.
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Web Designing</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>As a Senior Frontend Developer at USDT0, you will play a key role in building and refining our user-facing products. You’ll work closely with designers, product managers, and backend engineers to create intuitive, high-performing, and scalable web applications that showcase the potential of stablecoins to a global audience.
 This is a high-impact opportunity for someone passionate about building exceptional user experiences, solving complex problems, and advancing the adoption of stablecoins across industries.
 You will primarily be working on our consumer-facing applications, UI SDKs, and internal tooling. These surfaces combined will be responsible for moving and monitoring billions of dollars in transactions.
 WHAT YOU'LL DO
@@ -1032,9 +1726,18 @@
 Collaborative Culture: Join a team that values creativity, innovation, and shared success, with minimal bureaucracy and maximum ownership.
 This is your opportunity to lead frontend development at USDT0 and contribute to a project that is transforming how USDT empowers people worldwide.
 Join us in expanding access to financial stability for millions, ensuring that anyone, anywhere, can rely on the world’s most trusted digital dollar. Be part of building tools that make a meaningful difference for real people in high-inflation economies and unbanked communities across the globe.</t>
-  </si>
-  <si>
-    <t>Job Title: Senior Front End Developer (Crypto Focus)
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Web Designing</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Job Title: Senior Front End Developer (Crypto Focus)
 Employment Type: Full-Time (Paid in Crypto)
 Compensation: $80,000 - $110,000 per year
 Company Overview:
@@ -1079,9 +1782,18 @@
 Opportunity to make a significant impact in a small, focused team.
 Collaborative and innovative work environment, free from micromanagement.
 Please provide a cover letter with links to your previous portfolio work when applying</t>
-  </si>
-  <si>
-    <t>We're looking for passionate developers who love clean code, TDD and pair programming. If you are someone who spends his/her spare time on open source projects, keep up to date on the latest developments and techniques in the web based communication world, and love to hack on cool new projects, then keep reading!
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Web Designing</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>We're looking for passionate developers who love clean code, TDD and pair programming. If you are someone who spends his/her spare time on open source projects, keep up to date on the latest developments and techniques in the web based communication world, and love to hack on cool new projects, then keep reading!
 We are looking for software development interns to join the Commud gang for both 6 and 8 months terms.
 Your day at Commud
 Start your day at 9 am
@@ -1093,9 +1805,18 @@
 Become a smart mobile application developer.
 Constantly keep up to date with the latest news and techniques in the programming &amp; design.
 Be rewarded by your peers for your latest &amp; greatest work through our unique bonus system.</t>
-  </si>
-  <si>
-    <t>WHO YOU’LL WORK WITH
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Web Designing</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>WHO YOU’LL WORK WITH
 You will be part of the Global Technology organization and report to the Engineering Manager. On a daily basis, you will collaborate with peer software engineers, product managers, and architects onproduct teams to achieve business objectives. Additionally, you will engage with other Global Technology teams to align on both organizational and individual development goals.
 WHO WE ARE LOOKING FOR
 We are seeking a ambitious Full Stack Software Engineer to join our dynamic team. You’ll be responsible for developing and maintaining both front-end and back-end applications, ensuring seamless and scalable experiences for users. You will play a critical role in building robust features, maintaining system performance, and collaborating across teams to deliver high-quality cloud native software solutions. If you thrive in a collaborative environment, are energized by innovative technology, and excel at problem-solving, this role may be a great fit for you.
@@ -1124,9 +1845,18 @@
 Performance Optimization: Identify and fix performance bottlenecks across the full stack, ensuring high availability and responsiveness.
 CI/CD Integration: Integrate with and maintain continuous integration/continuous deployment (CI/CD) pipelines for seamless software delivery.
 Agile Methodologies: Participate in Agile processes, including sprint planning, daily stand-ups, code reviews, and retrospectives.</t>
-  </si>
-  <si>
-    <t>We are seeking an experienced Senior Full Stack Developer with strong expertise in React and Python to join our dynamic development team. In this role, you will design, develop, and maintain scalable web applications, leveraging your proficiency in React for front-end development, Python for back-end logic, and full-stack architecture. You’ll collaborate with cross-functional teams to deliver high-quality, user-focused solutions, utilizing modern tools including AI-powered coding assistants like Cursor. If you’re a problem-solver passionate about clean code and cutting-edge technologies, we’d love to hear from you!
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Web Designing</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>We are seeking an experienced Senior Full Stack Developer with strong expertise in React and Python to join our dynamic development team. In this role, you will design, develop, and maintain scalable web applications, leveraging your proficiency in React for front-end development, Python for back-end logic, and full-stack architecture. You’ll collaborate with cross-functional teams to deliver high-quality, user-focused solutions, utilizing modern tools including AI-powered coding assistants like Cursor. If you’re a problem-solver passionate about clean code and cutting-edge technologies, we’d love to hear from you!
 Key Responsibilities:
 Design and implement responsive, high-performance front-end applications using React.js, ensuring seamless user experiences.
 Develop and maintain robust back-end systems using Python frameworks (e.g., Django, Flask, or FastAPI) to support business logic and APIs.
@@ -1159,9 +1889,18 @@
 Experience:
 full-stack web development with a focus on React and Python: 3 years (Required)
 Application Deadline: 07/03/2025</t>
-  </si>
-  <si>
-    <t>Key Responsibilities:
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Web Designing</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Key Responsibilities:
 Team Leadership:
 Lead and manage a team of graphic designers, providing direction, feedback, and support to ensure the creation of high-quality design solutions.
 Foster a positive, collaborative, and creative work environment that encourages innovation and excellence.
@@ -1211,9 +1950,18 @@
 Location:
 Vaishali Nagar, Jaipur, Rajasthan (Required)
 Work Location: In person</t>
-  </si>
-  <si>
-    <t>WHO YOU’LL WORK WITH
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Web Designing</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>WHO YOU’LL WORK WITH
 You will be part of the Global Technology organization and report to the Engineering Manager. On a daily basis, you will collaborate with peer software engineers, product managers, and architects on product teams to achieve business objectives. Additionally, you will engage with other Global Technology teams to align on both organizational and individual development goals.
 WHO WE ARE LOOKING FOR
 We are seeking a ambitious Lead Full Stack Software Engineer to join our dynamic team. You’ll be responsible for developing and maintaining both front-end and back-end applications, ensuring seamless and scalable experiences for users. You will play a critical role in building robust features, maintaining system performance, and collaborating across teams to deliver high-quality cloud native software solutions. If you thrive in a collaborative environment, are energized by innovative technology, and excel at problem-solving, this role may be a great fit for you.
@@ -1258,12 +2006,18 @@
 Agile Methodologies: Participate in Agile processes, including sprint planning, daily stand-ups, code reviews, and retrospectives.
 Provide technical leadership and mentorship to your teammates and develop a team environment that promotes collaboration and innovation
 Contribute to existing documentation or educational content and adapt content based on product/program updates and user feedback.</t>
-  </si>
-  <si>
-    <t>Java Developer</t>
-  </si>
-  <si>
-    <t>Job description : Dear Candidate, We had an opportunity as Jr Java Developer-Chennai
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Java Developer</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Job description : Dear Candidate, We had an opportunity as Jr Java Developer-Chennai
 Hands on experience in designing and developing applications using Java EE platforms
 Object oriented analysis and design using common design patterns.
 Excellent knowledge of Relational Databases Oracle, SQL Server, SQL
@@ -1273,9 +2027,18 @@
 Experience in Conducting code reviews and mentor team members
 Good Communication, interpersonal and leadership skills
 Insurance Domain Knowledge is a plus If interested than kindly send your updated profile at prachi@busisol.net Thanks</t>
-  </si>
-  <si>
-    <t>Come work at a place where innovation and teamwork come together to support the most exciting missions in the world!
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Java Developer</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Come work at a place where innovation and teamwork come together to support the most exciting missions in the world!
 We are seeking a highly motivated and talented Software Engineer to work on Qualys’ next-generation data platform and middleware. Working alongside a very talented team of engineers and architects, you will be responsible for prototyping, designing, developing and supporting a highly scalable SaaS based cloud security data platform. This is a great opportunity to be an integral part of a team building Qualys’ next generation microservices based technology platform processing over a 100 million transactions and terabytes of data per day, leverage open source technologies, and work on challenging and business-impacting projects.
 Responsibilities
 As a data platform engineer you will be responsible for the team running data stored with millions of transactions per second, scaling 100s of terrabytes of data. Responsible for driving the data source and providing data platform as a service to all applications built in Qualys.
@@ -1330,9 +2093,18 @@
 Experience with configuration management tools such as Chef, Puppet or Ansible.
 In-depth experience with continuous integration and continuous deployment pipelines.
 Exposure to Maven, Ant or Gradle for builds.</t>
-  </si>
-  <si>
-    <t>Greetings from TCS!!!
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Java Developer</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Greetings from TCS!!!
 **TCS is Hiring for Java Developer**
 Desired Experience: 4-7 Years
 Job Location: Bhubaneshwar/Kolkata/Pune
@@ -1343,9 +2115,18 @@
 Knowledge and hands on experience on REST API, DB2, Github, TestNG/Junit, Selenium Technologies
 Good functional analysis skill
 Good team skill and communication skill</t>
-  </si>
-  <si>
-    <t>About the job
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Java Developer</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>About the job
 We are looking for a highly skilled Java Developer to join our team. The ideal candidate should have expertise in Java 8+, Spring Boot, and Microservices, with experience in building scalable and high-performance applications. The role involves end-to-end development, debugging, testing, and collaborating with teams to deliver quality solutions.
 Job Title: Java Developer
 Experience: 5 to 8 years
@@ -1375,9 +2156,18 @@
 We have been certified as a Great Place to Work® company for two consecutive years (2020-2022) and voted as the Top 20 AI/ML vendor by CIO Insider.
 Over the years, Wissen Group has successfully delivered multi million worth of projects for more than 20 of the Fortune 500 companies. Wissen Technology provides exceptional value in mission critical projects for its clients, through thought leadership, ownership, and assured on-time deliveries that are always ‘first time right’.
 The technology and thought leadership that the company commands in the industry is the direct result of the kind of people Wissen has been able to attract. Wissen is committed to providing them the best possible opportunities and careers, which extends to providing the best possible experience and value to our clients. We serve clients across sectors like Banking, Ecommerce, Telecom, Healthcare, Manufacturing, and Energy.</t>
-  </si>
-  <si>
-    <t>Job Title: Java Developer (AWS Cloud, DSA)
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Java Developer</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Job Title: Java Developer (AWS Cloud, DSA)
 Experience: 4+ Years
 Location: Hyderabad
 Job Type: Full-Time
@@ -1399,9 +2189,18 @@
 Preferred Qualifications:
 AWS certifications (AWS Certified Developer – Associate).
 Knowledge of SQL/NoSQL databases, Redis/Memcached, and Agile methodologies.</t>
-  </si>
-  <si>
-    <t>Minimum Qualifications:
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Java Developer</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Minimum Qualifications:
 Completed bachelor’s degree in Computer Science, Computer Engineering, Math or other Science major
 Excellent verbal and written communication skills
 Ability to research and execute solutions based on online guides and tutorials
@@ -1452,9 +2251,18 @@
 8 hour shift
 Monday to Friday
 Work Location: In person</t>
-  </si>
-  <si>
-    <t>Location:
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Java Developer</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Location:
 Tempa/ Charlotte, Irving Multiple USA
 Duration:
 Long Term
@@ -1469,9 +2277,18 @@
 Proficiency in front-end technologies (React/Angular, JavaScript).
 Hands-on experience with cloud platforms (AWS/Azure).
 Familiarity with databases like MySQL, PostgreSQL, or MongoDB.</t>
-  </si>
-  <si>
-    <t>Your Impact
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Java Developer</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Your Impact
 As a Software Engineer for Lowe’s, you’ll be transforming business needs into innovative software solutions. You will use a variety of computing environments to help us develop and deploy logical applications, from building intuitive UI to developing microservices with cloud-native technologies. The creative solutions you build will be able to impact thousands of our customers and associates daily.
 Work with a Winning Team
 As part of a Fortune 50 company and retail leader, your work can change an entire industry. Our CEO is a forward-thinker when it comes to tech, and with one of Forbes Top 50 CIOs leading the charge, you can come to work knowing you’ll have access to the data, tools, and support that few other companies can offer. We also know what it takes to create an inclusive culture that supports you.
@@ -1505,9 +2322,18 @@
 Lowe’s Companies, Inc. (NYSE: LOW) is a FORTUNE® 50 home improvement company serving approximately 16 million customer transactions a week in the United States. With total fiscal year 2023 sales of more than $86 billion, Lowe’s operates over 1,700 home improvement stores and employs approximately 300,000 associates. Based in Mooresville, N.C., Lowe’s supports the communities it serves through programs focused on creating safe, affordable housing and helping to develop the next generation of skilled trade experts. For more information, visit Lowes.com.
 Lowe’s is an equal opportunity employer and administers all personnel practices without regard to race, color, religious creed, sex, gender, age, ancestry, national origin, mental or physical disability or medical condition, sexual orientation, gender identity or expression, marital status, military or veteran status, genetic information, or any other category protected under federal, state, or local law.
 Pay Range: $75,300.00 - $143,100.00 annually Starting rate of pay may vary based on factors including, but not limited to, position offered, location, education, training, and/or experience. For information regarding our benefit programs and eligibility, please visit https://talent.lowes.com/us/en/benefits.</t>
-  </si>
-  <si>
-    <t>Overview
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Java Developer</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Overview
 As an integral part of our agile development team, you will develop and maintain our customer-facing web application. Using your analytical and problem-solving skills, you will work independently to solve complex problems. In our agile development process, you will work collaboratively with stakeholders and contribute ideas toward continuous process improvement. You will find plenty of opportunities to use and grow your abilities.
 What You Do:
 You will translate business requirements and bug reports into working solutions while minimizing technical debt
@@ -1580,9 +2406,18 @@
 If you have a disability or impairment and need assistance with the application process, please email recruiting@payscale.com for support.
 Fraud Alert:
 Payscale values security and privacy. During your job application and interview process, we will never ask for your personal banking or financial information, social security number, or other sensitive information, if you are unsure if a message is from Payscale, please email recruiting@payscale.com</t>
-  </si>
-  <si>
-    <t>Type: Full-Time
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Java Developer</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Type: Full-Time
 Primary Location: US
 Education: Bachelor’s Degree
 Salary Range: $115,000-$175,000
@@ -1619,9 +2454,18 @@
 4 X Mid or Junior Level Java Engineers with 2-5 years of experience
 We’d love to hear from you if you’re passionate about building scalable, user-focused solutions and thrive in a fast-paced, collaborative setting. Join us to shape the future of technology and make a lasting impact!
 Prospect 33 is an Equal Employment Opportunity/Affirmative Action Employer. We are a diverse and inclusive company. Great talent is always welcome at Prospect 33 regardless of background, ethnicity, race, gender, sexual orientation, religious views, or even political views.</t>
-  </si>
-  <si>
-    <t>About ComPsych:
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Java Developer</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>About ComPsych:
 ComPsych® Corporation is the world’s largest provider of mental health services and GuidanceResources® for life. Fueled by a commitment to relentless innovation and a comprehensive approach to care, ComPsych provides services to more than 78,000 organizations and 163 million individuals across 200 countries. Under our GuidanceResources® brand, our personalized and fully integrated programs include behavioral health, absence management, and wellness journeys, which empower employees to lead healthier and more productive lives, while driving organizational excellence. Visit compsych.com to find out why 40% of the Fortune 500 choose ComPsych for their mental health needs.
 Job Summary:
 We are currently looking for a self-motivated full-stack software developer to join our Business Applications Team. Our Business Applications team develops web applications and back-end business processes to help our coworkers assist clients with life concerns. In this role, as an individual contributor, you’ll be involved in many aspects – helping to design and architect technical solutions, innovating and collaborating with a high-performing technical team, and of course performing hands-on development for our new features and functionality.
@@ -1652,9 +2496,18 @@
 Competitive pay with annual increases
 EEO
 ComPsych celebrates diversity and is an equal opportunity employer. All applicants will be considered for employment regardless of race, color, age, genetics, religion, gender, sexual orientation, gender identity, national origin, disability or protected veteran status and any other characteristic protected by federal, state or local laws. ComPsych Corporation maintains a drug free workplace.</t>
-  </si>
-  <si>
-    <t>NOW HIRING
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Java Developer</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>NOW HIRING
 JUNIOR DEVELOPER - REMOTE
 ABOUT US
 Blue Cloud is the largest pediatric Ambulatory Surgery Center (ASC) company in the country, specializing in dental restorative and exodontia surgery for pediatric and special needs patients delivered under general anesthesia. We are a mission-driven company with an emphasis on providing safe, quality, and accessible care, at reduced costs to families and payors.
@@ -1695,9 +2548,18 @@
 Work with a passionate, dedicated, and talented team in a growing organization committed to doing good
 401k plan, including company match
 Blue Cloud is an equal opportunity employer. Consistent with applicable law, all qualified applicants will receive consideration for employment without regard to age, ancestry, citizenship, color, family or medical care leave, gender identity or expression, genetic information, immigration status, marital status, medical condition, national origin, physical or mental disability, political affiliation, protected veteran or military status, race, ethnicity, religion, sex (including pregnancy), sexual orientation, or any other characteristic protected by applicable local laws, regulations and ordinances. If you need assistance and/or a reasonable accommodation due to a disability during the application process, read more about requesting accommodations.</t>
-  </si>
-  <si>
-    <t>Job Title: Senior Software Engineer
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Java Developer</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Job Title: Senior Software Engineer
 Location: Remote
 Who We Are
 HMH is a learning technology company committed to delivering connected solutions that engage learners, empower educators, and improve student outcomes. As a leading provider of K–12 core curriculum, supplemental and intervention solutions and professional learning services, HMH partners with educators and school districts to uncover solutions that unlock students' potential and extend teachers' capabilities. HMH serves more than 50 million students and 4 million educators in 150 countries.
@@ -1729,9 +2591,18 @@
 The application window for this position is anticipated to close on March 31, 2025 . We encourage you to apply as soon as possible. The posting may be available past this date but is not guaranteed.
 HMH is fully committed to Equal Employment Opportunity and to attracting, retaining, developing and promoting the most qualified employees without regard to race, gender, color, religion, sexual orientation, family status, marital status, pregnancy, gender identity, ethnic/national origin, ancestry, age, disability, military status, genetic predisposition, citizenship status, status as a disabled veteran, recently separated veteran, Armed Forces service medal veteran, other covered veteran, or any other characteristic protected by federal, state or local law. We are dedicated to providing a work environment free from discrimination and harassment, and where employees are treated with respect and dignity. We actively participate in E-Verify.
 #LI-VA1</t>
-  </si>
-  <si>
-    <t>Wipro Limited (NYSE: WIT, BSE: 507685, NSE: WIPRO) is a leading technology services and consulting company focused on building innovative solutions that address clients’ most complex digital transformation needs. Leveraging our holistic portfolio of capabilities in consulting, design, engineering, and operations, we help clients realize their boldest ambitions and build future-ready, sustainable businesses. With over 230,000 employees and business partners across 65 countries, we deliver on the promise of helping our customers, colleagues, and communities thrive in an ever-changing world. For additional information, visit us at www.wipro.com.
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Java Developer</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Wipro Limited (NYSE: WIT, BSE: 507685, NSE: WIPRO) is a leading technology services and consulting company focused on building innovative solutions that address clients’ most complex digital transformation needs. Leveraging our holistic portfolio of capabilities in consulting, design, engineering, and operations, we help clients realize their boldest ambitions and build future-ready, sustainable businesses. With over 230,000 employees and business partners across 65 countries, we deliver on the promise of helping our customers, colleagues, and communities thrive in an ever-changing world. For additional information, visit us at www.wipro.com.
 Fullstack Java Developer
 Location: Irving, Texas(Fulltime role)
 Deep understanding of Object-Oriented Principles and Java, as well as broad cross-functional knowledge including relational and NoSQL database, software security, system administration, and enterprise messaging patterns.
@@ -1746,9 +2617,18 @@
 Experience with UI using REACTJS, AngularJS etc.
 Expected annual pay for this role ranges from $60,000 to $1,35,000 . Based on the position, the role is also eligible for Wipro’s standard benefits including a full range of medical and dental benefits options, disability insurance, paid time off (inclusive of sick leave), other paid and unpaid leave options.
 Wipro is an Equal Employment Opportunity employer and makes all employment and employment-related decisions without regard to a person's race, sex, national origin, ancestry, disability, sexual orientation, or any other status protected by applicable law.</t>
-  </si>
-  <si>
-    <t>Position ID
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Java Developer</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Position ID
 Java
 Job Title
 Java/UI Developer
@@ -1769,9 +2649,41 @@
 Bachelorâ€™s degree in Computer Science or a closely related field
 Location
 USA</t>
-  </si>
-  <si>
-    <t>Our Mission
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Java Developer</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>We're looking for passionate developers who love clean code, TDD and pair programming. If you are someone who spends his/her spare time on open source projects, keep up to date on the latest developments and techniques in the web based communication world, and love to hack on cool new projects, then keep reading!
+We are looking for software development interns to join the Commud gang for both 6 and 8 months terms.
+Your day at Commud
+Start your day at 9 am
+Do pair programming with another great developer on cool new upcoming features.
+Collaborate with a designer to make your feature look world-class.
+Participate in talk about the latest programming languages, tools and frameworks with other developers.
+What you Get
+Become a master in Java, HTML5, Ruby and web development.
+Become a smart mobile application developer.
+Constantly keep up to date with the latest news and techniques in the programming &amp; design.
+Be rewarded by your peers for your latest &amp; greatest work through our unique bonus system.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Java Developer</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Our Mission
 As the world’s number 1 job site*, our mission is to help people get jobs. We strive to cultivate an inclusive and accessible workplace where all people feel comfortable being themselves. We're looking to grow our teams with more people who share our enthusiasm for innovation and creating the best experience for job seekers.
 (*Comscore, Total Visits, March 2024)
 Day to Day
@@ -1814,9 +2726,18 @@
 Application Question(s):
 Please note, that the following question will not impact your eligibility for the the role. Will you be able to attend an in-person interview during the interview process at the following location, Skyview Building 10, Floor 10 Survey No. 83/1 Raidurg (Panmaktha) Village, Rangareddi Hyderabad 500081, Telangana, India?
 Work Location: Remote</t>
-  </si>
-  <si>
-    <t>Software Principal Engineer
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Java Developer</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Software Principal Engineer
 The Software Engineering team delivers next-generation application enhancements and new products for a changing world. Working at the cutting edge, we design and develop software for platforms, peripherals, applications and diagnostics — all with the most advanced technologies, tools, software engineering methodologies and the collaboration of internal and external partners.
 Join us to do the best work of your career and make a profound social impact as a Software Principal Engineer on our Software Engineering Team in Bangalore.
 What you’ll achieve
@@ -1843,9 +2764,18 @@
 Application closing date: 21 March 2025
 Dell Technologies is committed to the principle of equal employment opportunity for all employees and to providing employees with a work environment free of discrimination and harassment. Read the full Equal Employment Opportunity Policy here.
 Job ID:R263253</t>
-  </si>
-  <si>
-    <t>Amex GBT is a place where colleagues find inspiration in travel as a force for good and – through their work – can make an impact on our industry. We’re here to help our colleagues achieve success and offer an inclusive and collaborative culture where your voice is valued.
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Java Developer</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Amex GBT is a place where colleagues find inspiration in travel as a force for good and – through their work – can make an impact on our industry. We’re here to help our colleagues achieve success and offer an inclusive and collaborative culture where your voice is valued.
 Ready to explore a career path? Start your journey.
 What You’ll do on a Typical Day:
 We are looking for a highly motivated, self-driven, self-starter and fast-growing potential individual to be part of a growing team of technologists.
@@ -1890,9 +2820,18 @@
 All applicants will receive equal consideration for employment without regard to age, sex, gender (and characteristics related to sex and gender), pregnancy (and related medical conditions), race, color, citizenship, religion, disability, or any other class or characteristic protected by law.
 Furthermore, we are committed to providing reasonable accommodation to qualified individuals with disabilities. Please let your recruiter know if you need an accommodation at any point during the hiring process. For details regarding how we protect your data, please consult GBT Recruitment Privacy Statement.
 What if I don’t meet every requirement? If you’re passionate about our mission and believe you’d be a phenomenal addition to our team, don’t worry about “checking every box;" please apply anyway. You may be exactly the person we’re looking for!</t>
-  </si>
-  <si>
-    <t>Optum is a global organization that delivers care, aided by technology to help millions of people live healthier lives. The work you do with our team will directly improve health outcomes by connecting people with the care, pharmacy benefits, data and resources they need to feel their best. Here, you will find a culture guided by diversity and inclusion, talented peers, comprehensive benefits and career development opportunities. Come make an impact on the communities we serve as you help us advance health equity on a global scale. Join us to start Caring. Connecting. Growing together.
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Java Developer</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Optum is a global organization that delivers care, aided by technology to help millions of people live healthier lives. The work you do with our team will directly improve health outcomes by connecting people with the care, pharmacy benefits, data and resources they need to feel their best. Here, you will find a culture guided by diversity and inclusion, talented peers, comprehensive benefits and career development opportunities. Come make an impact on the communities we serve as you help us advance health equity on a global scale. Join us to start Caring. Connecting. Growing together.
 #GEN
 Primary Responsibilities:
 Involve in critical and complex technical discussions
@@ -1914,12 +2853,18 @@
 Proven ability to prioritize and manage work to critical project timelines in a fast-paced environment
 Proven detail-oriented and ability to document low to highly complex functional designs and data structures, to support business and operational requirement
 At UnitedHealth Group, our mission is to help people live healthier lives and make the health system work better for everyone. We believe everyone–of every race, gender, sexuality, age, location and income–deserves the opportunity to live their healthiest life. Today, however, there are still far too many barriers to good health which are disproportionately experienced by people of color, historically marginalized groups and those with lower incomes. We are committed to mitigating our impact on the environment and enabling and delivering equitable care that addresses health disparities and improves health outcomes — an enterprise priority reflected in our mission.</t>
-  </si>
-  <si>
-    <t>DevOps Engineer</t>
-  </si>
-  <si>
-    <t>Company Overview
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Company Overview
 At Motorola Solutions, we're guided by a shared purpose - helping people be their best in the moments that matter - and we live up to our purpose every day by solving for safer. Because people can only be their best when they not only feel safe, but are safe. We're solving for safer by building the best possible technologies across every part of our safety and security ecosystem. That's mission -critical communications devices and networks, AI-powered video security &amp; access control and the ability to unite voice, video and data in a single command center view. We're solving for safer by connecting public safety agencies and enterprises, enabling the collaboration that's critical to connect those in need with those who can help. The work we do here matters.
 Department Overview
 The Junior DevOps Engineer will be an integral member of the IT operations team, working closely with Cloud Operations, development, QA, and IT teams to facilitate the smooth deployment and operation of infrastructure, on-prem and software. The role involves learning and assisting with the automation of the software delivery process, ensuring scalable and efficient development cycles, and maintaining the infrastructure necessary for optimal system performance.
@@ -1956,9 +2901,18 @@
 Motorola Solutions is an Equal Opportunity Employer. All qualified applicants will receive consideration for employment without regard to race, color, religion or belief, sex, sexual orientation, gender identity, national origin, disability, veteran status or any other legally-protected characteristic.
 We are proud of our people-first and community-focused culture, empowering every Motorolan to be their most authentic self and to do their best work to deliver on the promise of a safer world. If you’d like to join our team but feel that you don’t quite meet all of the preferred skills, we’d still love to hear why you think you’d be a great addition to our team.
 We’re committed to providing an inclusive and accessible recruiting experience for candidates with disabilities, or other physical or mental health conditions. To request an accommodation, please email ohr@motorolasolutions.com.</t>
-  </si>
-  <si>
-    <t>About the job
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>About the job
 Support and deploy mission-critical, customer-facing, frontend and back-end production SaaS environments
  Improve site performance, monitoring, and overall stability of the production environments
  Performance tuning, monitoring, maintaining faulttolerant/HA infrastructure Disaster recovery, design implementation and maintenance
@@ -1968,9 +2922,18 @@
  Build documentation of operating procedures and train junior team member
 Desired Skills and Experience
 devops, AWS, AZURE, Linux 2 administration, RDBMS, nosql</t>
-  </si>
-  <si>
-    <t>About the Role:
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>About the Role:
 Are you a talented and motivated Network DevOps Engineer looking for an exciting remote opportunity? Join our dynamic team and be part of a cutting-edge network automation project. We are seeking a skilled professional with strong coding and support skills to help reduce alerts and ticket volumes, land bug-fixes, and support various automation workflows.
 Key Responsibilities:
 Automation and Troubleshooting: Develop and support automated system recovery tooling, prioritize alert failures, and aggregate failures for consolidated reporting.
@@ -1996,9 +2959,18 @@
 Level 1: $6.18/hr. to $9.26/hr. (USD) or 529/hr to 729/hr (INR)
 Exact compensation may vary based on several factors, including skills, experience, and education.
 Benefit packages for this role will start on the 31st day of employment and include medical, dental, and vision insurance.</t>
-  </si>
-  <si>
-    <t>Greetings from TCS!!!
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Greetings from TCS!!!
 **TCS is Hiring for AWS DevOps Engineer**
 Role: AWS DevOps Engineer
 Desired Experience: 4- 8 Years
@@ -2013,9 +2985,18 @@
 Create and maintain platform/services automation documentation support
 Provide support for projects prior to transition phase to support
 AWS Cloud services; Azure Cloud services: Terraform: Kubernetes: Docker containers: Python (or Go-lang): shell scripting network services: CI/CD pipelines and tools; cyber security standards and tools (e.g., secrets management, IAM)</t>
-  </si>
-  <si>
-    <t>Job Description
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Job Description
 Experience:
 Should have 4+ years of relevant experience in Database &amp; Operations (DBOps).
 Skillset/Technologies:
@@ -2033,9 +3014,18 @@
 Database Administration, Operations support for production/lower environment 
 Handling any infrastructure-related issues and deploying RFCs. 
 Coordinating with the Dev team, SA team, QA team, and Hadoop team to ensure the smooth operation of applications.</t>
-  </si>
-  <si>
-    <t>By making evidence the heart of security, we help customers stay ahead of ever-changing cyber-attacks.
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>By making evidence the heart of security, we help customers stay ahead of ever-changing cyber-attacks.
 Corelight is a cybersecurity company that transforms network and cloud activity into evidence. Evidence that elite defenders use to proactively hunt for threats, accelerate response to cyber incidents, gain complete network visibility and create powerful analytics using machine-learning and behavioral analysis tools. Easily deployed, and available in traditional and SaaS-based formats, Corelight is the fastest-growing Network Detection and Response (NDR) platform in the industry. And we are the only NDR platform that leverages the power of Open Source projects in addition to our own technology to deliver Intrusion Detection (IDS), Network Security Monitoring (NSM), and Smart PCAP solutions. We sell to some of the most sensitive, mission critical large enterprises and government agencies in the world.
 As the Lead Software Engineer -Cloud Infrastructure you will collaborate with development and quality engineering to build and maintain our continuous integration pipeline from development to production. You’ll bring a strong systems background and an eye toward automated software engineering and continuous delivery. Your deep understanding of SaaS and cloud technologies, combined with your leadership skills, will be vital in shaping the future of Corelight's Open NDR SaaS Platform.
 Responsibilities:
@@ -2071,9 +3061,18 @@
 Familiarity with configuration management tools (e.g., Ansible, Puppet, Chef)
 We are proud of our culture and values - driving diversity of background and thought, low-ego results, applied curiosity and tireless service to our customers and community. Corelight is committed to a geographically dispersed yet connected employee base with employees working from home and office locations around the world. Fueled by an accelerating revenue stream, and investments from top-tier venture capital organizations such as Crowdstrike, Accel and Insight - we are rapidly expanding our team.
 www.corelight.com</t>
-  </si>
-  <si>
-    <t>T-Rex Solutions is looking to select a Cloud Network Engineer to support the US Department of the Treasury TCloud enterprise cloud development effort. This effort aims to facilitate holistic multi-cloud solutions to meet the Department of Treasury’s enterprise-wide infrastructure needs. This position will be responsible for managing the configuration, installation and on-going support of the Network Infrastructure which includes Palo Alto firewalls, Cisco VPN Concentrators, Cisco CSR devices as well as Networking in cloud platforms such as Azure and OCI. The candidate for this position should have extensive hands-on technical skills designing and deploying various network technologies in cloud platforms. The scope of this position includes network design, implementation, and support for all components within cloud platforms. This position will need to be adept at monitoring the ongoing operation of the network and identifying potential issues and corrective actions as needed.
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>T-Rex Solutions is looking to select a Cloud Network Engineer to support the US Department of the Treasury TCloud enterprise cloud development effort. This effort aims to facilitate holistic multi-cloud solutions to meet the Department of Treasury’s enterprise-wide infrastructure needs. This position will be responsible for managing the configuration, installation and on-going support of the Network Infrastructure which includes Palo Alto firewalls, Cisco VPN Concentrators, Cisco CSR devices as well as Networking in cloud platforms such as Azure and OCI. The candidate for this position should have extensive hands-on technical skills designing and deploying various network technologies in cloud platforms. The scope of this position includes network design, implementation, and support for all components within cloud platforms. This position will need to be adept at monitoring the ongoing operation of the network and identifying potential issues and corrective actions as needed.
 Responsibilities:
 In-Depth knowledge and hands-on experience with major cloud platforms, such as Azure, OCI and GCP.
 Comprehensive knowledge of cloud security best practices and ability to implement security measures within cloud networks.
@@ -2108,9 +3107,18 @@
 T-Rex is an Equal Opportunity Employer. All qualified applicants will receive consideration for employment without regard to race, religion, color, sex (including pregnancy, gender identity, and sexual orientation), parental status, national origin, age, disability, family medical history or genetic information, political affiliation, military service, or other non-merit based factors.
 In compliance with pay transparency guidelines, the annual base salary range for this position is $100,000 - $130,000. Please note that the salary information is a general guideline only. T-Rex considers factors such as (but not limited to) scope and responsibilities of the position, candidate’s work experience, education/training, key skills, internal peer equity, as well as market and business considerations when extending an offer.
 T-Rex offers a diverse and collaborative work environment, exciting opportunities for professional growth, and generous benefits, including: PTO available to use immediately upon joining (prorated based on start date), paid parental leave, individual and family health, vision, and dental benefits, annual budget for training, professional development and tuition reimbursement, and a 401(k) plan with company match fully vested after 60 days of employment among other benefits.</t>
-  </si>
-  <si>
-    <t>Location: Remote | Full-Time
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Location: Remote | Full-Time
 Sequencing.com is looking for a Senior DevOps Engineer to join our growing Engineering team. This role is crucial to the daily development, deployment, and improvement of our large-scale technical infrastructure. We are a fast-paced startup where self-sufficiency, problem-solving, and ownership are highly valued. If you thrive in an environment where your expertise in DevOps, security, and automation will make a direct impact, we want to hear from you.
 Key Responsibilities
 Design, implement, and optimize DevOps processes for Sequencing.com’s large-scale technical suite.
@@ -2144,9 +3152,18 @@
 Sequencing makes Whole Genome Sequencing, the world's most comprehensive genetic testing, accessible and affordable. Our clinical-grade test and genetic analysis screens for over 15,000 conditions, providing deep insights into potential health risks. It translates genetic data into actionable steps to manage health and enhance well-being.
 Our user base is rapidly expanding, and the personal genomics market is experiencing unprecedented growth. We’re venture-backed and scaling rapidly to meet consumer demand.
 Sequencing.com is an equal opportunity employer. All aspects of employment, including the decision to hire, promote, discipline, or discharge, will be based on merit, competence, performance, and business needs. We do not discriminate based on race, color, religion, marital status, age, national origin, ancestry, physical or mental disability, medical condition, pregnancy, genetic information, gender, sexual orientation, gender identity or expression, veteran status, or any other status protected under federal, state, or local law.</t>
-  </si>
-  <si>
-    <t>Local or 100% Remote
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Local or 100% Remote
 Who we are
 Our mission at Point is to make homeownership more valuable and accessible to all. Every day, we explore, build, and iterate to create innovative financial products that improve the lives of our customers. Together, we’re creating the premier full-stack home equity platform to help current homeowners access their home wealth and aspiring ones realize their dream of homeownership. Point has raised over $180M from Andreessen Horowitz, WestCap, Prudential and other leading investors.
 About the role
@@ -2192,9 +3209,18 @@
 Tier 2 | Chicago, Austin, Denver, Boston, Washington DC, San Diego | $121,040 - $181,560
 Tier 3 | All other US metro areas | $113,920 - $170,880
 This does not include any other potential components of the compensation package, including equity, benefits, and perks outlined above. At the launch of each position, we benchmark compensation to the appropriate role and level utilizing competitive compensation data from various data sources as references. At the offer stage, we use the signal we received from our interviews coupled with your experience, location, and other job-related factors to determine final compensation.</t>
-  </si>
-  <si>
-    <t>Wunderkind is looking for a Senior Engineer to join our Professional Services team.
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Wunderkind is looking for a Senior Engineer to join our Professional Services team.
 We’re looking for a software engineer who is collaborative, eager to learn, and ready to make an impact. In this position you will play a critical role in delivering technical solutions and services for our clients. You will sit within a cross-functional Services team, working with clients to understand their needs and deliver customized engineering solutions.
 Responsibilities
 Own the process of scoping and implementing technical solutions, including third-party integrations with our client’s tech stack
@@ -2234,9 +3260,18 @@
 Proud to be an equal opportunity and safe workplace
 Strongly committed to equal employment opportunities for all races, colors, ancestries, national origins, marital statuses, age, citizenship, disabilities, genders or gender identities, or Veteran status
 The base salary range for this role is $95,000 to $115,000. Actual compensation packages are based on several factors that are unique to each specific candidate; including but not limited to skill set, depth of experience, applicable certifications, and geographic work location. This may vary depending on living location and market rate.</t>
-  </si>
-  <si>
-    <t>About the Position
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>About the Position
 The Senior Platform Engineer will report to the Lead DevOps Engineer. They will help pioneer industry-leading technologies and toolsets to enable our developers to innovate in record time. They will have the opportunity to create, evolve, scale, integrate, fortify, and automate our deployment pipeline and core services to solve unique and constantly-iterating engineering challenges.
 About the Core Platform Team
 The Core Platform team, inside the R&amp;D organization, is responsible for working with R&amp;D teams across the global FiscalNote organization. Core Platform is responsible for owning and evolving common tools, libraries, standards, and practices that are shared by numerous teams with similar needs. By understanding the team’s needs and leveraging best practices, Core Platform can become a force multiplier for the R&amp;D organization.
@@ -2266,9 +3301,18 @@
 Experience designing and developing CI/CD pipelines, preferably in Github Actions.
 Experience with Linux CLI and POSIX shells.
 Experience with working with multiple development teams on different projects.</t>
-  </si>
-  <si>
-    <t>A big hello from the team at Compuco!
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>A big hello from the team at Compuco!
 At Compuco we empower socially responsible organisations with the digital tools they need to build a better world.
 As a data driven creative technology agency, we are passionate about helping membership, charitable and cultural organisations to streamline and reimagine the way they work so that they can focus on impact.
 We’re on the lookout for an exceptional DevOps engineer to join our growing team. Your work will have a significant impact and the role will expose you to working on a range of open-source projects for the not-for-profit sector.
@@ -2321,9 +3365,18 @@
 Medical insurance allowance
 Paid leave for personal development and learning
 Remote working</t>
-  </si>
-  <si>
-    <t>Key Responsibilities:
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Key Responsibilities:
 Infrastructure Management:
 Configure and maintain Bastion Hosts for secure access to internal systems.
 Manage Amazon RDS for high-availability databases.
@@ -2356,9 +3409,18 @@
 Certification in AWS (e.g., AWS Certified DevOps Engineer).
 Experience with monitoring tools (e.g., Prometheus, Grafana).
 Familiarity with cost management tools like AWS Cost Explorer.</t>
-  </si>
-  <si>
-    <t>Company: Cognixus
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Company: Cognixus
 Position : Senior DevOps Engineer
 Location : Plaza Conlay, KL
 About the Company
@@ -2394,9 +3456,18 @@
 Practical knowledge of High Availability and distributed system Implementation using but not limited to Keepalived, etcd, zookeeper is an added advantages
 Practical Knowledge and understanding of DEVOPS, CI/CD (Git, GitLab, Gerrit, Jenkins, Harbor), Log Platform (ELK: Elasticsearch, Logstash/FileBeat, Kibana), Monitoring platform architecture technology (Zabbix / Prometheus) is an added advantage.
 Prior experience with Agile development methodology and Test-Driven development is an added advantage.</t>
-  </si>
-  <si>
-    <t>WHO WE ARE: MagicSchool is the premier generative AI platform for teachers. We're just over a year and a half old, and more than 4M teachers from all over the world have joined our platform. Join a top team at a fast growing company that is working towards real social impact. Make an account and try us out at our website and connect with our passionate community on our Wall of Love.
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>WHO WE ARE: MagicSchool is the premier generative AI platform for teachers. We're just over a year and a half old, and more than 4M teachers from all over the world have joined our platform. Join a top team at a fast growing company that is working towards real social impact. Make an account and try us out at our website and connect with our passionate community on our Wall of Love.
 Enterprise Cloud Architect
 Role Description: As an Enterprise Cloud Architect, you will design and implement scalable, secure, and innovative cloud solutions, enabling your organization to harness the full potential of AWS and Google Cloud. You will be a strategic partner to technical and business stakeholders, ensuring seamless integration of cloud services with enterprise needs while driving cost efficiency and performance.
 Responsibilities:
@@ -2433,9 +3504,18 @@
 Responsibility: Put responsibility and safety at the forefront of the technological change that AI is bringing to education.
 Diversity: Diversity of thought, perspectives, and backgrounds helps us serve the wide audience of educators and students around the world.
 Excellence: Educators and students deserve the best - and we strive for the highest quality in everything we do.</t>
-  </si>
-  <si>
-    <t>Job Description:
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Job Description:
 About Streamline:
 Streamline’s mission is to build innovative technology solutions that empower people who improve behavioral health and quality of life of those in need. We are a high growth technology company that delivers web-based software for healthcare organization’s to provide and coordinate all service delivery processes. Streamline has been offering software in the behavioral health marketplace since 2003. Streamline has built and maintains systems for some of the nation’s premier behavioral health organizations using the latest web-based technology. Streamline offers competitive compensation and benefits packages as well as a challenging, yet flexible, work environment that is conducive to collaboration and productivity. A career with Streamline Healthcare Solutions provides opportunities for growth and continued learning in a workplace where individual contribution is valued and recognized. Join us, and advance your career today with a company that is on the cutting edge of the behavioral healthcare technology industry. Here at Streamline, we strive on building lasting and trusting relationships with our clients, and our employees set the bar
 Requirement
@@ -2445,9 +3525,18 @@
 Qualification: BE/B.Tech/M. Tech/M. Sc and MCA
 Excellent verbal and written communication skills with extensive collaboration with US counterparts.
 Streamline Healthcare Solutions is an Equal Opportunity Employer. We celebrate diversity and are committed to creating an inclusive environment for all employees. Qualified applicants will receive consideration for employment without regard to race, color, religion, sex, age, disability, military status, national origin, or any other characteristic protected under federal, state, or applicable local law.</t>
-  </si>
-  <si>
-    <t>Company Overview
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Company Overview
 At Motorola Solutions, we're guided by a shared purpose - helping people be their best in the moments that matter - and we live up to our purpose every day by solving for safer. Because people can only be their best when they not only feel safe, but are safe. We're solving for safer by building the best possible technologies across every part of our safety and security ecosystem. That's mission -critical communications devices and networks, AI-powered video security &amp; access control and the ability to unite voice, video and data in a single command center view. We're solving for safer by connecting public safety agencies and enterprises, enabling the collaboration that's critical to connect those in need with those who can help. The work we do here matters.
 Department Overview
 The Junior DevOps Engineer will be an integral member of the IT operations team, working closely with Cloud Operations, development, QA, and IT teams to facilitate the smooth deployment and operation of infrastructure, on-prem and software. The role involves learning and assisting with the automation of the software delivery process, ensuring scalable and efficient development cycles, and maintaining the infrastructure necessary for optimal system performance.
@@ -2484,9 +3573,18 @@
 Motorola Solutions is an Equal Opportunity Employer. All qualified applicants will receive consideration for employment without regard to race, color, religion or belief, sex, sexual orientation, gender identity, national origin, disability, veteran status or any other legally-protected characteristic.
 We are proud of our people-first and community-focused culture, empowering every Motorolan to be their most authentic self and to do their best work to deliver on the promise of a safer world. If you’d like to join our team but feel that you don’t quite meet all of the preferred skills, we’d still love to hear why you think you’d be a great addition to our team.
 We’re committed to providing an inclusive and accessible recruiting experience for candidates with disabilities, or other physical or mental health conditions. To request an accommodation, please email ohr@motorolasolutions.com.</t>
-  </si>
-  <si>
-    <t>JOB DESCRIPTION
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>JOB DESCRIPTION
 Work with highly-skilled team of technologists who are responsible for maintaining JPMorgan’s cutting edge Trading applications. The platform provides services ranging from OMS, market data, reference data, session and recovery management, routing and back office system feeding for Global markets.
 As a Lead Software Engineer at JPMorgan Chase within the Commercial &amp; Investment Bank's Equities team, you will participate in all aspects of e-trading development from design and build to deployment with a focus on infrastructure, administrative, operational tasks as detailed in Key Responsibilities. You must be comfortable working as a front-office specialist in a high pressure, challenging environment and solving business and development tasks via technology in a fast pace: time to market is critical, but without compromising on quality or performance.
 Job Responsibilities
@@ -2509,9 +3607,18 @@
 Experience with GIT, Jira, Confluence, Wiki
 Experience in using Jenkins pipelines and building CI/CD pipelines.
 ABOUT US</t>
-  </si>
-  <si>
-    <t>Introduction
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Introduction
 As a DevOps engineer, you will work as an integral part of our Agile development team as well as Operations team, to deliver reliable and robust services to our board customer base. You will be involved in every stage of the development process and take pride in delivering great new services with excellent reliability. You will bring onboard a strong sense of ownership and will thrive in a fast-paced production environment.
 Roles &amp; Responsibilities:
 Understanding customer requirements and project KPIs
@@ -2539,9 +3646,18 @@
 MRI Software is a global Proptech leader delivering innovative applications and hosted solutions that free real estate companies to elevate their business.
 Our flexible technology platform, along with an open and connected ecosystem, allows us to meet the unique needs of real estate businesses, from property-level management and accounting to investment modeling and analytics for the global commercial and residential markets. With nearly five decades of expertise and insight, we have grown to include offices across the United States, the United Kingdom, Hong Kong, Singapore, Australia, South Africa, New Zealand, Canada, and India, with over 3500 team members to support our clients and their unique needs!
 MRI is proud to be an Equal Employment Opportunity employer.</t>
-  </si>
-  <si>
-    <t>Welcome to Warner Bros. Discovery… the stuff dreams are made of.
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Welcome to Warner Bros. Discovery… the stuff dreams are made of.
 Who We Are…
 When we say, “the stuff dreams are made of,” we’re not just referring to the world of wizards, dragons and superheroes, or even to the wonders of Planet Earth. Behind WBD’s vast portfolio of iconic content and beloved brands, are the storytellers bringing our characters to life, the creators bringing them to your living rooms and the dreamers creating what’s next…
 From brilliant creatives, to technology trailblazers, across the globe, WBD offers career defining opportunities, thoughtfully curated benefits, and the tools to explore and grow into your best selves. Here you are supported, here you are celebrated, here you can thrive.
@@ -2586,12 +3702,18 @@
 Championing Inclusion at WBD
 Warner Bros. Discovery embraces the opportunity to build a workforce that reflects the diversity of our society and the world around us. Being an equal opportunity employer means that we take seriously our responsibility to consider qualified candidates on the basis of merit, regardless of sex, gender identity, ethnicity, age, sexual orientation, religion or belief, marital status, pregnancy, parenthood, disability or any other category protected by law.
 If you’re a qualified candidate with a disability and you require adjustments or accommodations during the job application and/or recruitment process, please visit our accessibility page for instructions to submit your request.</t>
-  </si>
-  <si>
-    <t>Database</t>
-  </si>
-  <si>
-    <t>What Success Looks Like In This Role
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>What Success Looks Like In This Role
  Team member
  Learning processes and tools.
  Escalate issues as and when required.
@@ -2617,9 +3739,18 @@
  Excellent written and verbal communication skills with good command over English language.
 Unisys is proud to be an equal opportunity employer that considers all qualified applicants without regard to age, blood type, caste, citizenship, color, disability, family medical history, family status, ethnicity, gender, gender expression, gender identity, genetic information, marital status, national origin, parental status, pregnancy, race, religion, sex, sexual orientation, transgender status, veteran status or any other category protected by law.
 This commitment includes our efforts to provide for all those who seek to express interest in employment the opportunity to participate without barriers. If you are a US job seeker unable to review the job opportunities herein, or cannot otherwise complete your expression of interest, without additional assistance and would like to discuss a request for reasonable accommodation, please contact our Global Recruiting organization at GlobalRecruiting@unisys.com or alternatively Toll Free: 888-560-1782 (Prompt 4). US job seekers can find more information about Unisys’ EEO commitment here.</t>
-  </si>
-  <si>
-    <t>Job Type: Full-Time
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Job Type: Full-Time
 Industry: Audience profiling, Analytics, Ad Tech, Streaming
 Company size: 11-50
 Company type: Private
@@ -2642,12 +3773,30 @@
 Collaborative office space available in WeWork, Bellandur.
 If you've read all the way to the bottom of this description, thank you for your interest in Streamhub!
 We are committed to equal employment opportunities regardless of race, colour, ancestry, religion, sex, national origin, sexual orientation, age, citizenship, marital status, disability, gender, gender identity or expression, or veteran status. We are proud to be an equal opportunity workplace.</t>
-  </si>
-  <si>
-    <t>P2-C2-STSUS shift till 11 PM ISTPrimary Skillsdata architecture for all AWS data servicesETL processes to load data into the data warehouseAthena, Python code, GlueLambda, DMS , RDS, Redshift Cloud FormationWrite SQL queries to support data analysis and reportingreports and dashboards to visualize dataJDSeeking a developer who has good Experience in Athena, Python code, Glue, Lambda, DMS , RDS, Redshift Cloud Formation and other AWS serverless resources. Can optimize data models for performance and efficiency. Able to write SQL queries to support data analysis and reportingResponsibilityDesign, implement, and maintain the data architecture for all AWS data servicesWork with stakeholders to identify business needs and requirements for data-related projectsDesign and implement ETL processes to load data into the data warehouseGood Experience in Athena, Python code, Glue, Lambda, DMS , RDS, Redshift Cloud Formation and othe</t>
-  </si>
-  <si>
-    <t>Qualifications 
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>P2-C2-STSUS shift till 11 PM ISTPrimary Skillsdata architecture for all AWS data servicesETL processes to load data into the data warehouseAthena, Python code, GlueLambda, DMS , RDS, Redshift Cloud FormationWrite SQL queries to support data analysis and reportingreports and dashboards to visualize dataJDSeeking a developer who has good Experience in Athena, Python code, Glue, Lambda, DMS , RDS, Redshift Cloud Formation and other AWS serverless resources. Can optimize data models for performance and efficiency. Able to write SQL queries to support data analysis and reportingResponsibilityDesign, implement, and maintain the data architecture for all AWS data servicesWork with stakeholders to identify business needs and requirements for data-related projectsDesign and implement ETL processes to load data into the data warehouseGood Experience in Athena, Python code, Glue, Lambda, DMS , RDS, Redshift Cloud Formation and othe</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Qualifications 
 Bachelor’s degree in Engineering or related field or relevant work experience
 3-4 years of Experience in Production Operations / Support area
 Should have worked on supporting BigData-related Ops/ Support preferably with Hadoop Map-Reduce background
@@ -2662,9 +3811,18 @@
 Leverage in-depth knowledge of architecture and data models to prevent or resolve issues
 Perform root-cause analysis &amp; come up with preventive actions
 Share knowledge within team through mentorships, coaching, technical talks and blogs</t>
-  </si>
-  <si>
-    <t>Hi,
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Hi,
 Below is the JD for Azure Data Engineer role. Please go through it and do let me know if you are interested.
 Role: Azure DE
 Location: Remote
@@ -2689,9 +3847,18 @@
 TAG Team
 Loc. 3 Cube Towers, F93C+X29, White Field Rd, Whitefield’s, HITEC City, Kondapur, Telangana 500081
 www.spaplc.com</t>
-  </si>
-  <si>
-    <t>Title: Principal Data Engineer
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Title: Principal Data Engineer
 Location: Remote - United States Only
 About InMarket
 Since 2010, InMarket has been the leader in 360-degree consumer intelligence and real-time activation for thousands of today’s top brands. Through InMarket's data-driven marketing platform, brands can build targeted audiences, activate media in real time, and measure success in driving return on ad spend. InMarket's proprietary Moments offering outperforms traditional mobile advertising by 6x.* Our LCI attribution platform, which won the MarTech Breakthrough Award for Best Advertising Measurement Platform, was validated by Forrester to drive an average of $40 ROAS for our clients.
@@ -2738,9 +3905,18 @@
 Actual salaries will vary depending on factors including but not limited to work experience, specialized skills and training, performance in role, business needs, and job requirements. Base salary is subject to change and may be modified in the future. Base salary is just one component of InMarket’s total rewards package that also may include bonus, equity, and benefits. Ask your recruiter for more information!
 At InMarket we are committed to a culture that supports diversity, inclusion, belonging and equal opportunity. We celebrate all people and believe everyone deserves respect regardless of race, gender, sexual orientation, backgrounds, experiences, abilities or beliefs.
 InMarket is an Equal Opportunity Employer (EOE). Qualified applicants are considered for employment without regard to age, race, color, religion, sex, national origin, sexual orientation, disability, or veteran status.</t>
-  </si>
-  <si>
-    <t>The Data Product team collaborates with an experienced group of data scientists, engineers, and product managers to build highly scalable features that power TRM's products and services. As a Staff Software Engineer on the Data Product team, you will be responsible for designing and building mission-critical data services. These features analyze and provide insights into blockchain transaction activity at petabyte scale, and ultimately work to build a safer financial system for billions of people..
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>The Data Product team collaborates with an experienced group of data scientists, engineers, and product managers to build highly scalable features that power TRM's products and services. As a Staff Software Engineer on the Data Product team, you will be responsible for designing and building mission-critical data services. These features analyze and provide insights into blockchain transaction activity at petabyte scale, and ultimately work to build a safer financial system for billions of people..
 The impact you’ll have here:
 Build highly scalable features that integrate with dozens of blockchains.
 Design and architect intricate data models for optimal storage and retrieval to support sub-second latency for querying blockchain data.
@@ -2774,9 +3950,18 @@
 The following represents the expected range of compensation for this role:
 The estimated base salary range for this role is $240,000 - $265,000.
 Additionally, this role may be eligible to participate in TRM’s equity plan.</t>
-  </si>
-  <si>
-    <t>Job Title: Senior Data Engineer
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Job Title: Senior Data Engineer
 Department: Technology
 About the Role:
 Join our dynamic team of talented engineers with a proven track record in constructing data warehouses, lakes, and pipelines. We are on a mission to fuel Unite Us' ongoing expansion and enhance its positive influence on both the healthcare industry and individuals nationwide. As part of our team, your role will be instrumental in collecting, processing, and delivering data to both internal and external stakeholders. This pivotal work empowers us to intelligently invest in emerging opportunities, quantifying the value and ROI that Unite Us networks bring to our customers. By leveraging your expertise, you will help establish Unite Us as a thought leader in the dynamic social care landscape. Become an integral part of our team and help us in shaping the future of healthcare and making a meaningful impact on the lives of people across the country.
@@ -2834,9 +4019,18 @@
 As part of this work at home job, we will provide you with all the necessary equipment to perform your duties, including a computer, mouse, keyboard as well as other items on our approved list of WFH supplies.
 Unite Us is committed to building a diverse team and fostering an inclusive culture, and is proud to be an equal opportunity employer. We embrace and encourage our employees' differences in race, religion, color, national origin, gender, family status, sexual orientation, gender identity, gender expression, age, veteran status, disability, pregnancy, medical conditions, and other characteristics. If you require assistance in applying for open positions due to a disability please email us at peopleops@uniteus.com to request an accommodation.
 #LI-Remote</t>
-  </si>
-  <si>
-    <t>Altinity is looking for database geeks able to guide users around the globe in building ClickHouse applications. We serve a rapidly expanding customer base as well as the broader ClickHouse open source community.
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Altinity is looking for database geeks able to guide users around the globe in building ClickHouse applications. We serve a rapidly expanding customer base as well as the broader ClickHouse open source community.
 Your responsibilities will be divided as follows:
 Support (75% of time)
 Helping build production-grade systems based on ClickHouse: advise how to design schemas, plan clusters etc. Environments range from single node setups to clusters with 100s of nodes, including Altinity.Cloud, our managed ClickHouse service.
@@ -2873,9 +4067,18 @@
 *NOTE: Experience with ClickHouse is a MUST for this position. *
 Please make sure you describe your experience with Clickhouse in your resume.
 We will not consider candidates who don't have experience with Clickhouse or don't mention this experience in their resume</t>
-  </si>
-  <si>
-    <t>The Opportunity:
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>The Opportunity:
 To help scale the world’s #1 system for self-improvement. As a Senior Analytics Engineer at GrowthDay, you’ll play a critical role in designing, optimizing, and managing our data infrastructure to drive product-led growth and AI innovation. You'll build scalable, high-performance data solutions, ensuring seamless integration across platforms and empowering the organization with actionable insights. This role is perfect for someone passionate about data architecture and driving business impact through data-driven decisions
 What You Will Do In This Role:
 Optimize our data ecosystem across Snowflake, MongoDB, and DBT.
@@ -2905,9 +4108,18 @@
 Creative Thinkers - We continuously live outside the box, thinking about the look and feel, and the interconnections between everything.
 Driven - We show up every day, taking action vs getting stuck or avoiding, and embrace hard work with a smile.
 Passionate Advocates For Our Customers' Growth and Experience - The fundamental reason GrowthDay exists. It is our purpose!</t>
-  </si>
-  <si>
-    <t>About Bikky
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>About Bikky
 Restaurants are the heart of our communities - where we go to celebrate life’s memorable moments with those we love, and find comfort and familiarity in the world.
 But while the digital and data revolutions have transformed other parts of commerce and hospitality, restaurants haven’t had the same opportunity. The result has been an industry that’s - on average - had their profit margins shrink by 5x over the past 20 years.
 Bikky was founded on the belief that restaurants deserve the same access to data as the largest, most sophisticated businesses in the world. We believe that data can fundamentally transform the economic model of the entire restaurant industry - producing better businesses, more jobs, and stronger communities.
@@ -2943,9 +4155,18 @@
 Ability to participate in a 401k
 Bikky offers a hybrid working environment. For candidates in New York City, we have an office where the team works 3-4 times per week.
 Flexible vacation policy</t>
-  </si>
-  <si>
-    <t>About Us / Why Join?
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>About Us / Why Join?
 We are a rapidly growing crypto hedge fund, 2 years old, managing a 9-figure AUM, generating 200%+ annualized returns with a 4 Sharpe.
 Our team has grown to approximately 40 professionals across Trading &amp; Research, Technology, and Operations.
 As part of our growing team, you will play a pivotal role in designing and implementing robust data infrastructures that enable seamless research, analytical workflows, and effective trade ideation and execution. If you are an experienced data engineering leader with a passion for complex data systems, we want to hear from you!
@@ -2991,9 +4212,18 @@
 Prior experience in a trading or financial services environment.
 Familiarity with statistical and machine learning concepts.
 Strong understanding of data security and privacy standards.</t>
-  </si>
-  <si>
-    <t>Web Scraping &amp; Data Engineer (Remote, Freelance/Part-Time/Full-Time)
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Web Scraping &amp; Data Engineer (Remote, Freelance/Part-Time/Full-Time)
 About Us
 We are a data scraping and analytics company specializing in bulk data extraction for corporate clients. Our mission is to deliver high-quality, structured data solutions that empower businesses with actionable insights.
 To support our growth, we are seeking a Web Scraping Engineer to help extract, process, large-scale datasets while ensuring efficiency, compliance, and scalability.
@@ -3028,9 +4258,18 @@
 Resume or CV highlighting relevant experience
 A short response to: "What is the most complex scraping challenge you have solved, and how?"
 Apply now and be part of our growing data solutions team.</t>
-  </si>
-  <si>
-    <t>About the Staff Data Engineer at Headspace:
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>About the Staff Data Engineer at Headspace:
 At Headspace, our mission is to transform mental healthcare to improve the health and happiness of the world. Core to this mission is our ability to responsibly and ethically leverage data to provide personalized care to each of our members, meeting them where they are on the mental health continuum. We are seeking experienced engineers to come work on our data platform and pipelines. This is an incredible opportunity to participate in building out our modern data platform, working with a diverse and talented crew. In this role, you will work closely with our data science, data analytics and engineering teams to enable the entire company to bring personalized mental health and wellness to all our members.
 What you will do:
 Lead the Development of Scalable Data Infrastructure: Drive the architecture and implementation of cutting-edge pySpark data pipelines to ingest and transform diverse datasets into the organization’s data lake in a fault-tolerant, robust system.
@@ -3060,9 +4299,18 @@
 *As such, Headspace requests that individuals who have received coaching or clinical services at Headspace wait until their care with Headspace is complete before applying for a position. If someone with a Headspace account is hired for a position, please note their account will be deactivated and they will not be able to use Headspace services for the duration of their employment. *
 Further, if Headspace cannot find a role that fails to resolve an ethical issue associated with a dual relationship, Headspace may need to take steps to ensure ethical obligations are being adhered to, including a delayed start date or a potential leave of absence. Such steps would be taken to protect both the former member, as well as any relevant individuals from their care team, from impairment, risk of exploitation, or harm.
 For how how we will use the personal information you provide as part of the application process, please see: https://www.headspace.com/applicant-notice</t>
-  </si>
-  <si>
-    <t>At The Alter Office, we build with purpose. No fluff, no filler—just real impact. The AdTech industry is a mess of fragmented data, clunky integrations, and slow decision-making. We're here to fix that. If you're a Data Engineer who thrives on building scalable, intelligent systems, this is your chance to create something that actually works.
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>At The Alter Office, we build with purpose. No fluff, no filler—just real impact. The AdTech industry is a mess of fragmented data, clunky integrations, and slow decision-making. We're here to fix that. If you're a Data Engineer who thrives on building scalable, intelligent systems, this is your chance to create something that actually works.
 What You'll Do
 🚀 Own the Data Backbone – Design and optimize real-time data pipelines for our Customer Data Platform (CDP)
 🔗 Seamlessly Connect AdTech – Build integrations with Google Ads, Facebook Ads, and DSPs for real-time campaign insights
@@ -3076,9 +4324,18 @@
 ✅ Strong understanding of real-time data streaming and machine learning pipelines
 Why Us?
 We believe in building, shipping, and improving—fast. No unnecessary layers of approval, no bloated processes—just good engineering, meaningful work, and real impact on the future of AdTech. If you want to build something that actually matters, let's talk.</t>
-  </si>
-  <si>
-    <t>About Us
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>About Us
 BichpadiSampda is a leading provider of HR and data-driven solutions, helping businesses streamline their workforce management. We are looking for a passionate Software Engineer Intern to join our team and work on exciting projects that impact real-world businesses.
 Key Responsibilities
 Assist in developing and testing software applications.
@@ -3125,9 +4382,18 @@
 Performance bonus
 Yearly bonus
 Work Location: Remote</t>
-  </si>
-  <si>
-    <t>Database Admin I is involved w/ developing, implementing, &amp; maintaining data specs, designs, integration, testing, &amp; documentation under the supervision of the Ld Database Administrator. They implement &amp; maintain data specs, testing (e.g., scripts), &amp; documentation as specified by user requirements. The incumbent maintains database performance by applying tuning methodologies and monitoring performance, security, server config, &amp; data integrity as directed by the Ld Database Administrator.
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Database Admin I is involved w/ developing, implementing, &amp; maintaining data specs, designs, integration, testing, &amp; documentation under the supervision of the Ld Database Administrator. They implement &amp; maintain data specs, testing (e.g., scripts), &amp; documentation as specified by user requirements. The incumbent maintains database performance by applying tuning methodologies and monitoring performance, security, server config, &amp; data integrity as directed by the Ld Database Administrator.
 Principal Accountabilities:
 Addresses database issues as assigned utilizing ticket system.
 Collaborates with Lead Database Engineer to maintain database size and scalability by evaluating database performance and trends, as well as w/ other database engineers to create robust, scalable database structures &amp; queries.
@@ -3144,9 +4410,18 @@
 Important Notice: Recruitment fraud is on the rise, with scammers using misleading promises of job offers and interviews to solicit money and personal information from job seekers. CME Group adheres to established procedures designed to maintain trust, confidence and security throughout our recruitment process. Learn more
 here
 .</t>
-  </si>
-  <si>
-    <t>Entity:
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Entity:
 Technology
 Job Family Group:
 IT&amp;S Group
@@ -3191,9 +4466,18 @@
 Legal Disclaimer:
 We are an equal opportunity employer and value diversity at our company. We do not discriminate on the basis of race, religion, color, national origin, sex, gender, gender expression, sexual orientation, age, marital status, socioeconomic status, neurodiversity/neurocognitive functioning, veteran status or disability status. Individuals with an accessibility need may request an adjustment/accommodation related to bp’s recruiting process (e.g., accessing the job application, completing required assessments, participating in telephone screenings or interviews, etc.). If you would like to request an adjustment/accommodation related to the recruitment process, please contact us.
 If you are selected for a position and depending upon your role, your employment may be contingent upon adherence to local policy. This may include pre-placement drug screening, medical review of physical fitness for the role, and background checks.</t>
-  </si>
-  <si>
-    <t>Optum is a global organization that delivers care, aided by technology to help millions of people live healthier lives. The work you do with our team will directly improve health outcomes by connecting people with the care, pharmacy benefits, data and resources they need to feel their best. Here, you will find a culture guided by diversity and inclusion, talented peers, comprehensive benefits and career development opportunities. Come make an impact on the communities we serve as you help us advance health equity on a global scale. Join us to start Caring. Connecting. Growing together.
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Optum is a global organization that delivers care, aided by technology to help millions of people live healthier lives. The work you do with our team will directly improve health outcomes by connecting people with the care, pharmacy benefits, data and resources they need to feel their best. Here, you will find a culture guided by diversity and inclusion, talented peers, comprehensive benefits and career development opportunities. Come make an impact on the communities we serve as you help us advance health equity on a global scale. Join us to start Caring. Connecting. Growing together.
 We are seeking a senior Database Administrator to be an integral part of the DBA Operations team. Must have experience with multiple database platforms primarily for Mongodb/MSSQL in cloud and secondary support for NOSQL DBs like Cosmos.The senior DBA position plays a crucial role in the continuous delivery of our database operations. The successful candidate will have a track record of operational excellence managing large scale databases and at least 10+ years of hands-on experience. You will have excellent communication skills, a keen attention to detail and a passion for learning new technology and building high quality, scalable solutions.
 Primary Responsibilities:
 Design and implement fault-tolerant SQL Server and MongoDB solutions using highly availability patterns for scalability and stability in on-premises and in Cloud (Azure, AWS, GCP)
@@ -3235,9 +4519,18 @@
 Cloud certifications or an interest in pursuing certification
 #Exetech
 At UnitedHealth Group, our mission is to help people live healthier lives and make the health system work better for everyone. We believe everyone–of every race, gender, sexuality, age, location and income–deserves the opportunity to live their healthiest life. Today, however, there are still far too many barriers to good health which are disproportionately experienced by people of color, historically marginalized groups and those with lower incomes. We are committed to mitigating our impact on the environment and enabling and delivering equitable care that addresses health disparities and improves health outcomes - an enterprise priority reflected in our mission.</t>
-  </si>
-  <si>
-    <t>Entity:
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Entity:
 Technology
 Job Family Group:
 IT&amp;S Group
@@ -3309,12 +4602,18 @@
 Legal Disclaimer:
 We are an equal opportunity employer and value diversity at our company. We do not discriminate on the basis of race, religion, color, national origin, sex, gender, gender expression, sexual orientation, age, marital status, socioeconomic status, neurodiversity/neurocognitive functioning, veteran status or disability status. Individuals with an accessibility need may request an adjustment/accommodation related to bp’s recruiting process (e.g., accessing the job application, completing required assessments, participating in telephone screenings or interviews, etc.). If you would like to request an adjustment/accommodation related to the recruitment process, please contact us.
 If you are selected for a position and depending upon your role, your employment may be contingent upon adherence to local policy. This may include pre-placement drug screening, medical review of physical fitness for the role, and background checks.</t>
-  </si>
-  <si>
-    <t>Testing</t>
-  </si>
-  <si>
-    <t>Bhikaji Cama Place, New Delhi Software Tester Experience : 0.6 to 2 yrs Skills Required : Job Summary : The responsibilities of a Software Test Engineer can be:
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Bhikaji Cama Place, New Delhi Software Tester Experience : 0.6 to 2 yrs Skills Required : Job Summary : The responsibilities of a Software Test Engineer can be:
 Go through the software requirements and get clarifications on ones doubts
 Become familiar with the software under test and any other software related to it
 Understand the master test plan and/ or the project plan
@@ -3331,9 +4630,18 @@
 Update test automation based on the updated test cases
 Log own time in the project management software or time tracking system
 Report work progress and any problems faced to the Test Lead or Project Manager as required</t>
-  </si>
-  <si>
-    <t>Software Tester Responsibilities
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Software Tester Responsibilities
 Your role will vary depending on project requirements. You may join a project at the initial implementation stages to assess potential risks, or be brought on to a project midway through, when testing becomes a key requirement.
 Your Work Activities Are Likely To Include
 meeting with system users to understand the scope of projects
@@ -3366,9 +4674,18 @@
 the ability to work in a team and individually
 organizational skills with the capability of working towards tight deadlines
 a passion for technology.</t>
-  </si>
-  <si>
-    <t>Job Requisition ID #
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Job Requisition ID #
 25WD85018
 Position Overview
 As a QA Tester (AutoCAD / Revit) for the Autodesk App Store, the candidate will primarily be in a testing role with a focus on the quality assurance (QA) of applications submitted by third-party developers. The QA Tester (AutoCAD / Revit) will test third-party applications working with Autodesk products and ensuring they meet the requisite quality requirements before posting them to be downloaded by end users from the Autodesk App Store.
@@ -3408,9 +4725,18 @@
 We take pride in cultivating a culture of belonging and an equitable workplace where everyone can thrive. Learn more here: https://www.autodesk.com/company/diversity-and-belonging
 Are you an existing contractor or consultant with Autodesk? 
 Please search for open jobs and apply internally (not on this external site).</t>
-  </si>
-  <si>
-    <t>Job Title: Android Application Tester with Automation
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Job Title: Android Application Tester with Automation
 Location: Bangalore
 Job Type: Full-Time
 Notice Period: 0-15 days
@@ -3438,12 +4764,30 @@
 Knowledge of performance testing tools.
 Work Environment:
 Candidates should be ready for 5 days' work from office (WFO).</t>
-  </si>
-  <si>
-    <t>We are seeking a highly skilled and experienced Senior Consultant to join our dynamic team. As a Senior Consultant, you will be responsible for automating Android, WEB, and API tests using Webdriver.io TypeScript. You must have a Bachelor's degree in computer science, software engineering, or a comparable discipline, along with a minimum of 8 years of work experience. You will need to have exceptional analytical acumen and problem-solving prowess, as well as a thorough grasp of application functionalities, debugging, and test methodologies. A meticulous approach with a pledge to produce top tier software is essential for this role. Proficiency in API and GUI testing techniques is also required. Extensive experience with agile software development cycles, encompassing design through to deployment, is a must. Knowledge of TestRail and test case management experience are preferred. Additionally, experience with various DBs such as Oracle, MS SQL, SQL Lite, and SQL Express, as well as good communication and experience working directly with client teams, are highly desirable. This is a hybrid role, and you will be expected to work both remotely and on-site as needed.</t>
-  </si>
-  <si>
-    <t>About Us
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>We are seeking a highly skilled and experienced Senior Consultant to join our dynamic team. As a Senior Consultant, you will be responsible for automating Android, WEB, and API tests using Webdriver.io TypeScript. You must have a Bachelor's degree in computer science, software engineering, or a comparable discipline, along with a minimum of 8 years of work experience. You will need to have exceptional analytical acumen and problem-solving prowess, as well as a thorough grasp of application functionalities, debugging, and test methodologies. A meticulous approach with a pledge to produce top tier software is essential for this role. Proficiency in API and GUI testing techniques is also required. Extensive experience with agile software development cycles, encompassing design through to deployment, is a must. Knowledge of TestRail and test case management experience are preferred. Additionally, experience with various DBs such as Oracle, MS SQL, SQL Lite, and SQL Express, as well as good communication and experience working directly with client teams, are highly desirable. This is a hybrid role, and you will be expected to work both remotely and on-site as needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>About Us
 Every year, over 100 million renters navigate the renewal process—a critical moment often representing their biggest annual expense. Yet, this process is filled with inefficiencies, causing frustration for renters and property managers alike and driving high turnover rates.
 At Renew, we’re on a mission to transform the way property managers approach resident retention. We provide tools that do more than renew leases—they renew relationships, helping turn renters into loyal, long-term customers. The rental market is massive, with large institutions owning tens of millions of units across the U.S. However, renters often remain unaware of the value these portfolios can offer. That’s where we come in. We’re building software that tackles real challenges for apartment operators while creating a rental experience that strengthens connections and unlocks lasting value for everyone involved.
 Our team is made up of experienced professionals from leading real estate tech companies like Compass, Jetty, Updater, and Rent. Together, we’ve launched and scaled successful businesses, and we’re backed by top-tier investors, including Ribbit, Khosla, Founders Fund, TPG, and some of the most prominent names in real estate. Renew is growing rapidly, and we’re already working with some of the largest institutional real estate firms in the country.
@@ -3479,9 +4823,18 @@
 Collaborate with a tight-knit, engineering-driven team that values automation and efficiency.
 Leverage cutting-edge AI tools to enhance testing speed and accuracy.
 Competitive salary + equity in a growing startup.</t>
-  </si>
-  <si>
-    <t>Please note:
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Please note:
 We do not accept applications without a personalized note explaining your interest in and suitability for this particular role with us.
 Compensation varies based on the type of engagement. Independent contractors may have higher rates than employees due to differences in tax and benefit structures.
 Valory
@@ -3526,9 +4879,18 @@
 You will work on a unique software stack and product with a team of world-class software engineers, researchers, and product experts across multiple fields.
 You will collaborate with teams across crypto and our community of agent developers.
 You will redefine how developers build off-chain services in DeFi and long into web3’s future.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Los Angeles (Santa Monica) or Remote (NA timezones)
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Los Angeles (Santa Monica) or Remote (NA timezones)
 About Maximus
 Maximus (https://www.maximustribe.com/) is a mission-driven consumer health company that provides men with content, community, and clinical support to optimize them in mind and body. Maximus has raised $15M from top Silicon Valley VCs such as Founders Fund and 8VC as well as leading angel investors/operators from companies like Bulletproof, Tinder, Coinbase, Daily Stoic, &amp; Shopify.
 Maximus is building an advanced telemedicine platform to help men improve their mental and physical health. We iterate on our product rapidly and safely by applying continuous integration and code quality measurements, as well as TDD and pair programming when appropriate. We work collaboratively, emphasizing the productivity of the team first. We aim to deliver a robust, reliable system by using pragmatic, tried-and-true technologies. We hone our craft as engineers by applying advanced functional, data-oriented techniques that are appropriate to the problem.
@@ -3578,9 +4940,18 @@
 Extended options exercise window for loyal employees (3 months for every year of service; e.g. 1 year for 4+ year employees)
 Maximus is an equal opportunity employer, which not only includes standard protected categories, but the additional freedom from discrimination against your free speech and beliefs, as long as they are aligned with company values. We celebrate intellectual diversity.
 </t>
-  </si>
-  <si>
-    <t>Oversee the quality assurance process, implementing advanced testing methodologies and tools to ensure robust software products meet high standards of functionality and reliability.
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Oversee the quality assurance process, implementing advanced testing methodologies and tools to ensure robust software products meet high standards of functionality and reliability.
 Master’s or Bachelor’s degree in Computer Science or Engineering, or a related field.
 Must have 3+ years of experience in automated and manual testing.
 Must have experience in leading a team of QA Engineers.
@@ -3589,9 +4960,18 @@
 Proficient in deriving and executing functional end-to-end scenarios.
 Extensive experience in performance testing using JMeter or similar tools, deep expertise in end-to-end, UI, API, functional, and non-functional testing, and a robust foundation in test automation frameworks and tools.
 Must exhibit a knack for problem-solving, a keen eye for detail, exceptional communication skills, and a collaborative spirit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Location: Remote | Full-Time
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Location: Remote | Full-Time
 Sequencing.com is seeking a Senior QA Engineer with strong manual testing skills and a deep understanding of test automation. While the role primarily involves manual QA, we are looking for someone who has experience designing, developing, and maintaining automation test suites. The ideal candidate will have prior experience working in an e-commerce environment and be familiar with modern test automation stacks—with Playwright experience being a major plus. Mobile review and performance testing are crucial for this role.
 Key Responsibilities
 Ensure user requirements are satisfied, releases to production are defect-free, and systems/changes perform as expected without adversely impacting operations.
@@ -3633,9 +5013,18 @@
 Our user base is rapidly expanding, and the personal genomics market is experiencing unprecedented growth. We’re venture-backed and scaling rapidly to meet consumer demand.
 Sequencing.com is an equal opportunity employer. All aspects of employment, including the decision to hire, promote, discipline, or discharge, will be based on merit, competence, performance, and business needs. We do not discriminate based on race, color, religion, marital status, age, national origin, ancestry, physical or mental disability, medical condition, pregnancy, genetic information, gender, sexual orientation, gender identity or expression, veteran status, or any other status protected under federal, state, or local law.
 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">About Staple:
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">About Staple:
 Staple is a Singapore based AI company with subsidiaries in Asia and the UK. Staple is helping to build the future of work by developing technology to interpret, extract, process and reconcile data workflows across structured, semi-structured and unstructured sources.
 Staple’s primary product offers interprets and extracts data from documents, and then matches this data between sources, without the need for templates.
 Since incorporating in 2018, Staple has been backed by Delivery Hero, Entrepreneur First, 500 Startups, and has won awards and recognition from Ernst and Young, Accenture and Enterprise Singapore to name a few. Our customers represent some of the largest multinationals in Singapore, and some of the largest financial institutions worldwide.
@@ -3673,9 +5062,18 @@
 20 days of paid leave annually to help nurture work-life balance
 If you are a meticulous QA Tester with a passion for ensuring top-notch software quality and want to be a part of the AI revolution in document processing, we encourage you to apply. Join us in building robust and reliable solutions that transform how businesses handle documents and unlock new possibilities.
 </t>
-  </si>
-  <si>
-    <t>Do you want to help make the world safe from cyber attack?
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Do you want to help make the world safe from cyber attack?
 At Corelight, we believe that the best approach to cybersecurity risk starts with the network. Attackers can evade endpoint detection, firewalls and many other technologies - but they can’t avoid leaving digital footprints on the networks they traverse. Built on open-source innovations from Zeek, Suricata and YARA and refined through years of real-world use, Corelight transforms network footprints from physical, virtual and cloud networks into actionable insights. Our customers use these insights to speed incident response, proactively hunt for threats and stay in compliance with cybersecurity regulations.
 We are seeking an experienced performance test engineer to validate the performance, reliability and scalability of the Corelight network sensor with a focus on testing in virtual and cloud environments at scale. The sensors can be combined into fleets of sensors to cover the entire network. You’ll harness your skills and experience to isolate the origin of issues from Linux network processing to traffic mix through to detection packages and exporting. Provide dashboards and self-service tooling for collaborators to confirm results in a fully automated fashion. Let the statistical significance of the data direct the prioritization of your work. Feel strongly that the usefulness of our findings directly correlates into how well we can map the symptoms into real work impact.
 Tackle system performance issues: analyze and debug complex system performance issues, identify bottlenecks and optimize product/service performance to improve user experience.
@@ -3698,9 +5096,18 @@
 Today, Corelight is the fastest growing network detection and response platform in the industry, trusted to protect mission-critical assets in leading enterprises, government agencies, and research institutions worldwide. We are leading the way with AI-assisted workflows, machine learning models, cloud security and SaaS-based solutions to arm defenders with the tools and knowledge they need to disrupt cyber attacks. Our team of passionate innovators are dedicated to solving some of the toughest challenges in cybersecurity, while fostering a collaborative, inclusive, and growth-oriented culture. At Corelight, we are proud of our diversity of background and thought, and we’re united by our strong shared culture and the values we live by every day.
 We are proud of our culture and values - driving diversity of background and thought, low-ego results, applied curiosity and tireless service to our customers and community. Corelight is committed to a geographically dispersed yet connected employee base with employees working from home and office locations around the world. Fueled by an accelerating revenue stream, and investments from top-tier venture capital organizations such as Crowdstrike, Accel and Insight - we are rapidly expanding our team.
 We are looking forward to meeting you. Check us out at www.corelight.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">🚀What's the position?
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">🚀What's the position?
 We're looking for a dedicated Mobile Tester to join our growing team at Neybox. This is full-time, remote position for Neybox Digital, a leading mobile app studio with two in-house mobile apps. With our apps, our goal is to help everyone live a better, healthier life.
 💫What will I be working on?
 We have two apps Pillow (https://pillow.app) and Today (https://neybox.com/today). These are two well-established, health and fitness mobile apps with millions of users worldwide. We don't accept any client work. As a member of our team you role
@@ -3740,9 +5147,18 @@
 Just hit the button "Apply" button below!
 ⚠️ Please note that this is the only acceptable way to apply. All other ways of contacting Neybox about the position (social media, LinkedIn, email etc.), will result in immediate rejection.
 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">We are looking for a skilled QA Engineer + Automation Engineer who is passionate about quality and technology. In this role, you will be responsible for designing and implementing automated test frameworks, writing and executing test scripts, and working closely with our development team to ensure product quality at every stage of the development process.
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We are looking for a skilled QA Engineer + Automation Engineer who is passionate about quality and technology. In this role, you will be responsible for designing and implementing automated test frameworks, writing and executing test scripts, and working closely with our development team to ensure product quality at every stage of the development process.
 Key Responsibilities:
 Design, develop, and maintain automated test scripts and frameworks for web and mobile applications.
 Execute and manage automated test suites, and analyze results to identify issues and areas for improvement.
@@ -3764,9 +5180,18 @@
 Strong analytical and problem-solving skills, with attention to detail.
 Excellent communication skills and ability to work effectively in a team environment.
 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">⚠️ ONLY APPLY THROUGH OUR APPLICATION FORM: https://stack-influence.breezy.hr/p/78672347f7b7/apply 👈
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">⚠️ ONLY APPLY THROUGH OUR APPLICATION FORM: https://stack-influence.breezy.hr/p/78672347f7b7/apply 👈
 Stack Influence is a VC-funded creator marketplace app connecting eCommerce brands with everyday social media users. We are a high-growth, remote-first startup.
 You will report directly to the CTO on a small product and engineering team. We are looking for a hybrid, technical analyst that can understand and test a modern Javascript codebase while also performing business analyst duties.
 Salary is between $75-100k USD with equity potential.
@@ -3785,9 +5210,18 @@
 Bachelor’s degree in Computer Science, Engineering, Information Systems or a related field.
 ⚠️ ONLY APPLY THROUGH OUR APPLICATION FORM: https://stack-influence.breezy.hr/p/78672347f7b7/apply 👈
 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">QA Automation Intern:
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA Automation Intern:
 We provide virtual business process services to overseas clients and this position is to be part of the dedicated team which provides mortgage back-office services and software product development to Toorak Capital Partners https://www.toorakcapital.com/ from Mortgage Finance Industry.
 About Toorak Capital
 Toorak Capital Partners (“Toorak”) is an integrated capital provider and investment manager headquartered in Summit, NJ. Toorak partners with private lenders throughout the U.S. and the U.K. and has acquired over $7.5B in (20,000+) business purpose mortgage loans backed by residential, multifamily, and mixed-use properties. Toorakmanages all aspects of its investment portfolio using its dedicated internal team, including loan sourcing, pricing, underwriting, acquisition, capital markets (securitization/debt issuance) and asset management. With capital commitments from entities managed by KKR, a leading global investment firm, Toorak has revolutionized the way business purpose real estate lenders access capital. The firm was the first to link private lenders with institutional capital. Toorak has been recognized by NJBIZ as New Jersey’s #1 fastest growing company in 2019 and 2020 and has earned the #3 spot for the Fastest Growing Company in NYC Metropolitan Area by Crain’s New York Business.
@@ -3816,9 +5250,18 @@
 Stipend: Best in Industry
 SEND APPLICATION TO: resume@finacplus.com
 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">For more than 40 years, Accelya has been the industry’s partner for change, simplifying airline financial and commercial processes and empowering the air transport community to take better control of the future. Whether partnering with IATA on industry-wide initiatives or enabling digital transformation to simplify airline processes, Accelya drives the airline industry forward and proudly puts control back in the hands of airlines so they can move further, faster.
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For more than 40 years, Accelya has been the industry’s partner for change, simplifying airline financial and commercial processes and empowering the air transport community to take better control of the future. Whether partnering with IATA on industry-wide initiatives or enabling digital transformation to simplify airline processes, Accelya drives the airline industry forward and proudly puts control back in the hands of airlines so they can move further, faster.
 Assist in the development and execution of test plans and test cases for new system implementations.
 Perform functional, integration, and regression testing to validate new features and system changes.
 Document test results, report defects, and work with development teams to facilitate issue resolution.
@@ -3828,9 +5271,18 @@
 Contribute to process improvements by identifying and suggesting enhancements to QA practices.
 What does the future of the air transport industry look like to you? Whether you’re an industry veteran or someone with experience from other industries, we want to make your ambitions a reality!
 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arm has built the world’s most pervasive compute architecture, and we’ve led many of the technology revolutions that impact the day-to-day lives of people everywhere. The Future of Infrastructure is Built on Arm. Now we are building new software teams to take us to the next level. Technology built on Arm is all around us, from industrial and automotive applications, to the IoT, to the desktop and data center. ‘Wherever Computing Happens’, we need to enable Arm by providing software solutions that interface higher-level software stacks with the hardware itself.
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Arm has built the world’s most pervasive compute architecture, and we’ve led many of the technology revolutions that impact the day-to-day lives of people everywhere. The Future of Infrastructure is Built on Arm. Now we are building new software teams to take us to the next level. Technology built on Arm is all around us, from industrial and automotive applications, to the IoT, to the desktop and data center. ‘Wherever Computing Happens’, we need to enable Arm by providing software solutions that interface higher-level software stacks with the hardware itself.
 JOB OVERVIEW:
 Arm is seeking skilled, experienced, and highly motivated Software QA expert to join our Software Engineering group. As a member of the System Solutions team, you will have the opportunity to enable the evolution of Computing Infrastructure using Arm Neoverse Compute Subsystems. You will be working with a distributed team spread across multiple locations. Your primary responsibilities will include ensuring firmware developed for Arm Neoverse CSS platforms is product ready.
 RESPONSIBILITIES:
@@ -3861,9 +5313,18 @@
 Equal Opportunities at Arm
 Arm is an equal opportunity employer, committed to providing an environment of mutual respect where equal opportunities are available to all applicants and colleagues. We are a diverse organization of dedicated and innovative individuals, and don’t discriminate on the basis of race, color, religion, sex, sexual orientation, gender identity, national origin, disability, or status as a protected veteran.
 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Job description
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Job description
 About this role
 Are you interested in building innovative technology that crafts the financial markets? Do you like working at the speed of a startup, and solving some of the world’s most exciting challenges? Do you want to work with, and learn from, hands-on leaders in technology and finance?
 At BlackRock, we are looking for Software Engineers who like to innovate and solve sophisticated problems. We recognize that strength comes from diversity, and will embrace your outstanding skills, curiosity, and passion while giving you the opportunity to grow technically and as an individual.
@@ -3904,9 +5365,18 @@
 Job Requisition #
 R250686
 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Asteria Aerospace Ltd is a full-stack drone technology company providing actionable intelligence from aerial data. We develop deeply customized drone solutions for government and enterprise customers using our in-house hardware design, software development, and manufacturing capabilities. We have been a trusted partner to provide long-term and quality-focused drone products &amp; services to the defense &amp; homeland security, agriculture, oil &amp; gas, energy &amp; utilities, telecommunications, mining, and construction sectors. Our drone solutions protect borders and facilities, improve farm yields, inspect critical assets, and monitor construction sites using the power of aerial intelligence. Asteria Aerospace is a subsidiary of Jio Platforms Ltd, which is a majority-owned subsidiary of Reliance Industries Ltd.
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asteria Aerospace Ltd is a full-stack drone technology company providing actionable intelligence from aerial data. We develop deeply customized drone solutions for government and enterprise customers using our in-house hardware design, software development, and manufacturing capabilities. We have been a trusted partner to provide long-term and quality-focused drone products &amp; services to the defense &amp; homeland security, agriculture, oil &amp; gas, energy &amp; utilities, telecommunications, mining, and construction sectors. Our drone solutions protect borders and facilities, improve farm yields, inspect critical assets, and monitor construction sites using the power of aerial intelligence. Asteria Aerospace is a subsidiary of Jio Platforms Ltd, which is a majority-owned subsidiary of Reliance Industries Ltd.
 If drones excite and inspire you, we would love to have you as a part of our growing team of change-makers. Don’t simply watch the latest tech unfold, be a part of creating the future with us!
 Our Values
 1. Take Charge
@@ -3937,1298 +5407,10 @@
 Team Working Skills.
 Confidence
 </t>
-  </si>
-</sst>
-</file>
-
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-  </fonts>
-  <fills count="2">
-    <fill>
-      <patternFill patternType="none"/>
-    </fill>
-    <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-  </fills>
-  <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-  </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-  </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
-</styleSheet>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="44546A"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="ED7D31"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="FFC000"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4472C4"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="70AD47"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0563C1"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="954F72"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
-</a:theme>
-</file>
-
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B121"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="27.28515625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>2</v>
-      </c>
-      <c r="B8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>2</v>
-      </c>
-      <c r="B9" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>2</v>
-      </c>
-      <c r="B10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>2</v>
-      </c>
-      <c r="B11" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>2</v>
-      </c>
-      <c r="B12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>2</v>
-      </c>
-      <c r="B13" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>2</v>
-      </c>
-      <c r="B14" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>2</v>
-      </c>
-      <c r="B15" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>2</v>
-      </c>
-      <c r="B16" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>2</v>
-      </c>
-      <c r="B17" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>2</v>
-      </c>
-      <c r="B18" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>2</v>
-      </c>
-      <c r="B19" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>2</v>
-      </c>
-      <c r="B20" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>2</v>
-      </c>
-      <c r="B21" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>23</v>
-      </c>
-      <c r="B22" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>23</v>
-      </c>
-      <c r="B23" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>23</v>
-      </c>
-      <c r="B24" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>23</v>
-      </c>
-      <c r="B25" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>23</v>
-      </c>
-      <c r="B26" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>23</v>
-      </c>
-      <c r="B27" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>23</v>
-      </c>
-      <c r="B28" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>23</v>
-      </c>
-      <c r="B29" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>23</v>
-      </c>
-      <c r="B30" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>23</v>
-      </c>
-      <c r="B31" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>23</v>
-      </c>
-      <c r="B32" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>23</v>
-      </c>
-      <c r="B33" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>23</v>
-      </c>
-      <c r="B34" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>23</v>
-      </c>
-      <c r="B35" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>23</v>
-      </c>
-      <c r="B36" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>23</v>
-      </c>
-      <c r="B37" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>23</v>
-      </c>
-      <c r="B38" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>23</v>
-      </c>
-      <c r="B39" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>23</v>
-      </c>
-      <c r="B40" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>23</v>
-      </c>
-      <c r="B41" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>44</v>
-      </c>
-      <c r="B42" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>44</v>
-      </c>
-      <c r="B43" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>44</v>
-      </c>
-      <c r="B44" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>44</v>
-      </c>
-      <c r="B45" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>44</v>
-      </c>
-      <c r="B46" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>44</v>
-      </c>
-      <c r="B47" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>44</v>
-      </c>
-      <c r="B48" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>44</v>
-      </c>
-      <c r="B49" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>44</v>
-      </c>
-      <c r="B50" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>44</v>
-      </c>
-      <c r="B51" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>44</v>
-      </c>
-      <c r="B52" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>44</v>
-      </c>
-      <c r="B53" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>44</v>
-      </c>
-      <c r="B54" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>44</v>
-      </c>
-      <c r="B55" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>44</v>
-      </c>
-      <c r="B56" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>44</v>
-      </c>
-      <c r="B57" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>44</v>
-      </c>
-      <c r="B58" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>44</v>
-      </c>
-      <c r="B59" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>44</v>
-      </c>
-      <c r="B60" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>44</v>
-      </c>
-      <c r="B61" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>64</v>
-      </c>
-      <c r="B62" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>64</v>
-      </c>
-      <c r="B63" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>64</v>
-      </c>
-      <c r="B64" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>64</v>
-      </c>
-      <c r="B65" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>64</v>
-      </c>
-      <c r="B66" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>64</v>
-      </c>
-      <c r="B67" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>64</v>
-      </c>
-      <c r="B68" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>64</v>
-      </c>
-      <c r="B69" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>64</v>
-      </c>
-      <c r="B70" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>64</v>
-      </c>
-      <c r="B71" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>64</v>
-      </c>
-      <c r="B72" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
-        <v>64</v>
-      </c>
-      <c r="B73" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
-        <v>64</v>
-      </c>
-      <c r="B74" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
-        <v>64</v>
-      </c>
-      <c r="B75" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>64</v>
-      </c>
-      <c r="B76" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
-        <v>64</v>
-      </c>
-      <c r="B77" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
-        <v>64</v>
-      </c>
-      <c r="B78" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
-        <v>64</v>
-      </c>
-      <c r="B79" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
-        <v>64</v>
-      </c>
-      <c r="B80" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
-        <v>64</v>
-      </c>
-      <c r="B81" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
-        <v>85</v>
-      </c>
-      <c r="B82" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
-        <v>85</v>
-      </c>
-      <c r="B83" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
-        <v>85</v>
-      </c>
-      <c r="B84" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
-        <v>85</v>
-      </c>
-      <c r="B85" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
-        <v>85</v>
-      </c>
-      <c r="B86" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
-        <v>85</v>
-      </c>
-      <c r="B87" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
-        <v>85</v>
-      </c>
-      <c r="B88" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
-        <v>85</v>
-      </c>
-      <c r="B89" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
-        <v>85</v>
-      </c>
-      <c r="B90" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
-        <v>85</v>
-      </c>
-      <c r="B91" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
-        <v>85</v>
-      </c>
-      <c r="B92" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
-        <v>85</v>
-      </c>
-      <c r="B93" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
-        <v>85</v>
-      </c>
-      <c r="B94" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
-        <v>85</v>
-      </c>
-      <c r="B95" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
-        <v>85</v>
-      </c>
-      <c r="B96" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
-        <v>85</v>
-      </c>
-      <c r="B97" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
-        <v>85</v>
-      </c>
-      <c r="B98" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
-        <v>85</v>
-      </c>
-      <c r="B99" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
-        <v>85</v>
-      </c>
-      <c r="B100" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
-        <v>85</v>
-      </c>
-      <c r="B101" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
-        <v>106</v>
-      </c>
-      <c r="B102" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
-        <v>106</v>
-      </c>
-      <c r="B103" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A104" t="s">
-        <v>106</v>
-      </c>
-      <c r="B104" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
-        <v>106</v>
-      </c>
-      <c r="B105" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A106" t="s">
-        <v>106</v>
-      </c>
-      <c r="B106" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A107" t="s">
-        <v>106</v>
-      </c>
-      <c r="B107" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A108" t="s">
-        <v>106</v>
-      </c>
-      <c r="B108" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A109" t="s">
-        <v>106</v>
-      </c>
-      <c r="B109" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A110" t="s">
-        <v>106</v>
-      </c>
-      <c r="B110" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A111" t="s">
-        <v>106</v>
-      </c>
-      <c r="B111" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
-        <v>106</v>
-      </c>
-      <c r="B112" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
-        <v>106</v>
-      </c>
-      <c r="B113" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A114" t="s">
-        <v>106</v>
-      </c>
-      <c r="B114" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A115" t="s">
-        <v>106</v>
-      </c>
-      <c r="B115" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A116" t="s">
-        <v>106</v>
-      </c>
-      <c r="B116" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A117" t="s">
-        <v>106</v>
-      </c>
-      <c r="B117" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
-        <v>106</v>
-      </c>
-      <c r="B118" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
-        <v>106</v>
-      </c>
-      <c r="B119" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A120" t="s">
-        <v>106</v>
-      </c>
-      <c r="B120" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
-        <v>106</v>
-      </c>
-      <c r="B121" t="s">
-        <v>126</v>
+        </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>